<commit_message>
fixed progress bar, prepated insatallation bat file
</commit_message>
<xml_diff>
--- a/excelReport/page-load-report.xlsx
+++ b/excelReport/page-load-report.xlsx
@@ -425,13 +425,13 @@
         <v>https://www.softwebsolutions.com/custom-net-development-services/</v>
       </c>
       <c r="B2">
-        <v>6.95</v>
+        <v>8.4</v>
       </c>
       <c r="C2" t="str">
-        <v>5/5/2026, 3:22:35 pm</v>
+        <v>7/5/2026, 12:00:41 am</v>
       </c>
       <c r="D2" t="str">
-        <v>5/5/2026, 3:22:42 pm</v>
+        <v>7/5/2026, 12:00:49 am</v>
       </c>
       <c r="E2" t="str">
         <v>Success</v>
@@ -442,13 +442,13 @@
         <v>https://www.softwebsolutions.com/custom-software-development/</v>
       </c>
       <c r="B3">
-        <v>4.54</v>
+        <v>6.14</v>
       </c>
       <c r="C3" t="str">
-        <v>5/5/2026, 3:22:47 pm</v>
+        <v>7/5/2026, 12:00:55 am</v>
       </c>
       <c r="D3" t="str">
-        <v>5/5/2026, 3:22:52 pm</v>
+        <v>7/5/2026, 12:01:01 am</v>
       </c>
       <c r="E3" t="str">
         <v>Success</v>
@@ -459,13 +459,13 @@
         <v>https://www.softwebsolutions.com/customer-care-bot-development/</v>
       </c>
       <c r="B4">
-        <v>1.31</v>
+        <v>1.99</v>
       </c>
       <c r="C4" t="str">
-        <v>5/5/2026, 3:22:56 pm</v>
+        <v>7/5/2026, 12:01:09 am</v>
       </c>
       <c r="D4" t="str">
-        <v>5/5/2026, 3:22:58 pm</v>
+        <v>7/5/2026, 12:01:11 am</v>
       </c>
       <c r="E4" t="str">
         <v>Success</v>
@@ -476,13 +476,13 @@
         <v>https://www.softwebsolutions.com/customer-data-platform/</v>
       </c>
       <c r="B5">
-        <v>5.24</v>
+        <v>5.48</v>
       </c>
       <c r="C5" t="str">
-        <v>5/5/2026, 3:23:03 pm</v>
+        <v>7/5/2026, 12:01:18 am</v>
       </c>
       <c r="D5" t="str">
-        <v>5/5/2026, 3:23:08 pm</v>
+        <v>7/5/2026, 12:01:23 am</v>
       </c>
       <c r="E5" t="str">
         <v>Success</v>
@@ -493,13 +493,13 @@
         <v>https://www.softwebsolutions.com/dashboard-development-services/</v>
       </c>
       <c r="B6">
-        <v>5.11</v>
+        <v>5.25</v>
       </c>
       <c r="C6" t="str">
-        <v>5/5/2026, 3:23:14 pm</v>
+        <v>7/5/2026, 12:01:31 am</v>
       </c>
       <c r="D6" t="str">
-        <v>5/5/2026, 3:23:19 pm</v>
+        <v>7/5/2026, 12:01:36 am</v>
       </c>
       <c r="E6" t="str">
         <v>Success</v>
@@ -510,13 +510,13 @@
         <v>https://www.softwebsolutions.com/data-analytics-banking-dashboard/</v>
       </c>
       <c r="B7">
-        <v>4.27</v>
+        <v>4.73</v>
       </c>
       <c r="C7" t="str">
-        <v>5/5/2026, 3:23:25 pm</v>
+        <v>7/5/2026, 12:01:43 am</v>
       </c>
       <c r="D7" t="str">
-        <v>5/5/2026, 3:23:30 pm</v>
+        <v>7/5/2026, 12:01:48 am</v>
       </c>
       <c r="E7" t="str">
         <v>Success</v>
@@ -527,13 +527,13 @@
         <v>https://www.softwebsolutions.com/data-analytics-finance-dashboard/</v>
       </c>
       <c r="B8">
-        <v>0.93</v>
+        <v>1.43</v>
       </c>
       <c r="C8" t="str">
-        <v>5/5/2026, 3:23:35 pm</v>
+        <v>7/5/2026, 12:01:54 am</v>
       </c>
       <c r="D8" t="str">
-        <v>5/5/2026, 3:23:36 pm</v>
+        <v>7/5/2026, 12:01:55 am</v>
       </c>
       <c r="E8" t="str">
         <v>Success</v>
@@ -544,13 +544,13 @@
         <v>https://www.softwebsolutions.com/data-analytics-services/</v>
       </c>
       <c r="B9">
-        <v>4.97</v>
+        <v>4.39</v>
       </c>
       <c r="C9" t="str">
-        <v>5/5/2026, 3:23:43 pm</v>
+        <v>7/5/2026, 12:02:01 am</v>
       </c>
       <c r="D9" t="str">
-        <v>5/5/2026, 3:23:48 pm</v>
+        <v>7/5/2026, 12:02:06 am</v>
       </c>
       <c r="E9" t="str">
         <v>Success</v>
@@ -561,13 +561,13 @@
         <v>https://www.softwebsolutions.com/data-engineering-consulting-services/</v>
       </c>
       <c r="B10">
-        <v>1.39</v>
+        <v>4.46</v>
       </c>
       <c r="C10" t="str">
-        <v>5/5/2026, 3:23:54 pm</v>
+        <v>7/5/2026, 12:02:11 am</v>
       </c>
       <c r="D10" t="str">
-        <v>5/5/2026, 3:23:55 pm</v>
+        <v>7/5/2026, 12:02:16 am</v>
       </c>
       <c r="E10" t="str">
         <v>Success</v>
@@ -578,13 +578,13 @@
         <v>https://www.softwebsolutions.com/data-governance-services/</v>
       </c>
       <c r="B11">
-        <v>5.96</v>
+        <v>2.13</v>
       </c>
       <c r="C11" t="str">
-        <v>5/5/2026, 3:24:01 pm</v>
+        <v>7/5/2026, 12:02:22 am</v>
       </c>
       <c r="D11" t="str">
-        <v>5/5/2026, 3:24:07 pm</v>
+        <v>7/5/2026, 12:02:25 am</v>
       </c>
       <c r="E11" t="str">
         <v>Success</v>
@@ -595,13 +595,13 @@
         <v>https://www.softwebsolutions.com/data-integration-services/</v>
       </c>
       <c r="B12">
-        <v>2.11</v>
+        <v>1.42</v>
       </c>
       <c r="C12" t="str">
-        <v>5/5/2026, 3:24:13 pm</v>
+        <v>7/5/2026, 12:02:31 am</v>
       </c>
       <c r="D12" t="str">
-        <v>5/5/2026, 3:24:15 pm</v>
+        <v>7/5/2026, 12:02:33 am</v>
       </c>
       <c r="E12" t="str">
         <v>Success</v>
@@ -612,13 +612,13 @@
         <v>https://www.softwebsolutions.com/data-managed-services/</v>
       </c>
       <c r="B13">
-        <v>2.27</v>
+        <v>4.99</v>
       </c>
       <c r="C13" t="str">
-        <v>5/5/2026, 3:24:21 pm</v>
+        <v>7/5/2026, 12:02:39 am</v>
       </c>
       <c r="D13" t="str">
-        <v>5/5/2026, 3:24:23 pm</v>
+        <v>7/5/2026, 12:02:44 am</v>
       </c>
       <c r="E13" t="str">
         <v>Success</v>
@@ -629,13 +629,13 @@
         <v>https://www.softwebsolutions.com/data-migration-services/</v>
       </c>
       <c r="B14">
-        <v>1.42</v>
+        <v>4.52</v>
       </c>
       <c r="C14" t="str">
-        <v>5/5/2026, 3:24:30 pm</v>
+        <v>7/5/2026, 12:02:50 am</v>
       </c>
       <c r="D14" t="str">
-        <v>5/5/2026, 3:24:31 pm</v>
+        <v>7/5/2026, 12:02:55 am</v>
       </c>
       <c r="E14" t="str">
         <v>Success</v>
@@ -646,13 +646,13 @@
         <v>https://www.softwebsolutions.com/data-pipeline-automation-services/</v>
       </c>
       <c r="B15">
-        <v>1.95</v>
+        <v>1.58</v>
       </c>
       <c r="C15" t="str">
-        <v>5/5/2026, 3:24:40 pm</v>
+        <v>7/5/2026, 12:03:01 am</v>
       </c>
       <c r="D15" t="str">
-        <v>5/5/2026, 3:24:42 pm</v>
+        <v>7/5/2026, 12:03:03 am</v>
       </c>
       <c r="E15" t="str">
         <v>Success</v>
@@ -663,13 +663,13 @@
         <v>https://www.softwebsolutions.com/data-science-development/</v>
       </c>
       <c r="B16">
-        <v>1.72</v>
+        <v>9.58</v>
       </c>
       <c r="C16" t="str">
-        <v>5/5/2026, 3:24:50 pm</v>
+        <v>7/5/2026, 12:03:08 am</v>
       </c>
       <c r="D16" t="str">
-        <v>5/5/2026, 3:24:52 pm</v>
+        <v>7/5/2026, 12:03:18 am</v>
       </c>
       <c r="E16" t="str">
         <v>Success</v>
@@ -680,13 +680,13 @@
         <v>https://www.softwebsolutions.com/data-visualization-consulting/</v>
       </c>
       <c r="B17">
-        <v>1.16</v>
+        <v>6.92</v>
       </c>
       <c r="C17" t="str">
-        <v>5/5/2026, 3:25:01 pm</v>
+        <v>7/5/2026, 12:03:24 am</v>
       </c>
       <c r="D17" t="str">
-        <v>5/5/2026, 3:25:02 pm</v>
+        <v>7/5/2026, 12:03:31 am</v>
       </c>
       <c r="E17" t="str">
         <v>Success</v>
@@ -697,13 +697,13 @@
         <v>https://www.softwebsolutions.com/databricks-consulting-services/</v>
       </c>
       <c r="B18">
-        <v>6.3</v>
+        <v>1.04</v>
       </c>
       <c r="C18" t="str">
-        <v>5/5/2026, 3:25:09 pm</v>
+        <v>7/5/2026, 12:03:36 am</v>
       </c>
       <c r="D18" t="str">
-        <v>5/5/2026, 3:25:15 pm</v>
+        <v>7/5/2026, 12:03:37 am</v>
       </c>
       <c r="E18" t="str">
         <v>Success</v>
@@ -714,13 +714,13 @@
         <v>https://www.softwebsolutions.com/decision-intelligence-system/</v>
       </c>
       <c r="B19">
-        <v>1.11</v>
+        <v>4.84</v>
       </c>
       <c r="C19" t="str">
-        <v>5/5/2026, 3:25:21 pm</v>
+        <v>7/5/2026, 12:03:43 am</v>
       </c>
       <c r="D19" t="str">
-        <v>5/5/2026, 3:25:23 pm</v>
+        <v>7/5/2026, 12:03:47 am</v>
       </c>
       <c r="E19" t="str">
         <v>Success</v>
@@ -731,13 +731,13 @@
         <v>https://www.softwebsolutions.com/deep-learning-solutions/</v>
       </c>
       <c r="B20">
-        <v>2.42</v>
+        <v>3.89</v>
       </c>
       <c r="C20" t="str">
-        <v>5/5/2026, 3:25:29 pm</v>
+        <v>7/5/2026, 12:03:53 am</v>
       </c>
       <c r="D20" t="str">
-        <v>5/5/2026, 3:25:31 pm</v>
+        <v>7/5/2026, 12:03:57 am</v>
       </c>
       <c r="E20" t="str">
         <v>Success</v>
@@ -748,13 +748,13 @@
         <v>https://www.softwebsolutions.com/defect-detection-in-packaging/</v>
       </c>
       <c r="B21">
-        <v>0.99</v>
+        <v>5.27</v>
       </c>
       <c r="C21" t="str">
-        <v>5/5/2026, 3:25:37 pm</v>
+        <v>7/5/2026, 12:04:04 am</v>
       </c>
       <c r="D21" t="str">
-        <v>5/5/2026, 3:25:38 pm</v>
+        <v>7/5/2026, 12:04:10 am</v>
       </c>
       <c r="E21" t="str">
         <v>Success</v>
@@ -765,13 +765,13 @@
         <v>https://www.softwebsolutions.com/devops-consulting-services/</v>
       </c>
       <c r="B22">
-        <v>4.54</v>
+        <v>4.73</v>
       </c>
       <c r="C22" t="str">
-        <v>5/5/2026, 3:25:45 pm</v>
+        <v>7/5/2026, 12:04:16 am</v>
       </c>
       <c r="D22" t="str">
-        <v>5/5/2026, 3:25:49 pm</v>
+        <v>7/5/2026, 12:04:21 am</v>
       </c>
       <c r="E22" t="str">
         <v>Success</v>
@@ -785,10 +785,10 @@
         <v>0.98</v>
       </c>
       <c r="C23" t="str">
-        <v>5/5/2026, 3:25:55 pm</v>
+        <v>7/5/2026, 12:04:28 am</v>
       </c>
       <c r="D23" t="str">
-        <v>5/5/2026, 3:25:56 pm</v>
+        <v>7/5/2026, 12:04:29 am</v>
       </c>
       <c r="E23" t="str">
         <v>Success</v>
@@ -799,13 +799,13 @@
         <v>https://www.softwebsolutions.com/digital-supply-chain-solutions/</v>
       </c>
       <c r="B24">
-        <v>1.46</v>
+        <v>1.13</v>
       </c>
       <c r="C24" t="str">
-        <v>5/5/2026, 3:26:03 pm</v>
+        <v>7/5/2026, 12:04:35 am</v>
       </c>
       <c r="D24" t="str">
-        <v>5/5/2026, 3:26:04 pm</v>
+        <v>7/5/2026, 12:04:36 am</v>
       </c>
       <c r="E24" t="str">
         <v>Success</v>
@@ -816,13 +816,13 @@
         <v>https://www.softwebsolutions.com/digital-supply-chain/</v>
       </c>
       <c r="B25">
-        <v>6.69</v>
+        <v>1.15</v>
       </c>
       <c r="C25" t="str">
-        <v>5/5/2026, 3:26:10 pm</v>
+        <v>7/5/2026, 12:04:44 am</v>
       </c>
       <c r="D25" t="str">
-        <v>5/5/2026, 3:26:17 pm</v>
+        <v>7/5/2026, 12:04:45 am</v>
       </c>
       <c r="E25" t="str">
         <v>Success</v>
@@ -833,13 +833,13 @@
         <v>https://www.softwebsolutions.com/digital-transformation-consulting/</v>
       </c>
       <c r="B26">
-        <v>4.7</v>
+        <v>1.53</v>
       </c>
       <c r="C26" t="str">
-        <v>5/5/2026, 3:26:22 pm</v>
+        <v>7/5/2026, 12:04:51 am</v>
       </c>
       <c r="D26" t="str">
-        <v>5/5/2026, 3:26:27 pm</v>
+        <v>7/5/2026, 12:04:53 am</v>
       </c>
       <c r="E26" t="str">
         <v>Success</v>
@@ -850,13 +850,13 @@
         <v>https://www.softwebsolutions.com/edge-ai-solutions/</v>
       </c>
       <c r="B27">
-        <v>1.65</v>
+        <v>5.3</v>
       </c>
       <c r="C27" t="str">
-        <v>5/5/2026, 3:26:32 pm</v>
+        <v>7/5/2026, 12:04:59 am</v>
       </c>
       <c r="D27" t="str">
-        <v>5/5/2026, 3:26:34 pm</v>
+        <v>7/5/2026, 12:05:04 am</v>
       </c>
       <c r="E27" t="str">
         <v>Success</v>
@@ -867,13 +867,13 @@
         <v>https://www.softwebsolutions.com/enterprise-app-development/</v>
       </c>
       <c r="B28">
-        <v>1.18</v>
+        <v>1.72</v>
       </c>
       <c r="C28" t="str">
-        <v>5/5/2026, 3:26:40 pm</v>
+        <v>7/5/2026, 12:05:12 am</v>
       </c>
       <c r="D28" t="str">
-        <v>5/5/2026, 3:26:42 pm</v>
+        <v>7/5/2026, 12:05:14 am</v>
       </c>
       <c r="E28" t="str">
         <v>Success</v>
@@ -884,13 +884,13 @@
         <v>https://www.softwebsolutions.com/enterprise-data-management-services/</v>
       </c>
       <c r="B29">
-        <v>5.18</v>
+        <v>6.1</v>
       </c>
       <c r="C29" t="str">
-        <v>5/5/2026, 3:26:48 pm</v>
+        <v>7/5/2026, 12:05:19 am</v>
       </c>
       <c r="D29" t="str">
-        <v>5/5/2026, 3:26:53 pm</v>
+        <v>7/5/2026, 12:05:25 am</v>
       </c>
       <c r="E29" t="str">
         <v>Success</v>
@@ -901,13 +901,13 @@
         <v>https://www.softwebsolutions.com/enterprise-data-warehouse/</v>
       </c>
       <c r="B30">
-        <v>4.54</v>
+        <v>4.63</v>
       </c>
       <c r="C30" t="str">
-        <v>5/5/2026, 3:27:01 pm</v>
+        <v>7/5/2026, 12:05:31 am</v>
       </c>
       <c r="D30" t="str">
-        <v>5/5/2026, 3:27:05 pm</v>
+        <v>7/5/2026, 12:05:36 am</v>
       </c>
       <c r="E30" t="str">
         <v>Success</v>
@@ -918,13 +918,13 @@
         <v>https://www.softwebsolutions.com/fabric-consulting-services/</v>
       </c>
       <c r="B31">
-        <v>4.25</v>
+        <v>8.93</v>
       </c>
       <c r="C31" t="str">
-        <v>5/5/2026, 3:27:12 pm</v>
+        <v>7/5/2026, 12:05:42 am</v>
       </c>
       <c r="D31" t="str">
-        <v>5/5/2026, 3:27:16 pm</v>
+        <v>7/5/2026, 12:05:51 am</v>
       </c>
       <c r="E31" t="str">
         <v>Success</v>
@@ -935,13 +935,13 @@
         <v>https://www.softwebsolutions.com/face-recognition-services/</v>
       </c>
       <c r="B32">
-        <v>4.6</v>
+        <v>8.92</v>
       </c>
       <c r="C32" t="str">
-        <v>5/5/2026, 3:27:22 pm</v>
+        <v>7/5/2026, 12:05:56 am</v>
       </c>
       <c r="D32" t="str">
-        <v>5/5/2026, 3:27:27 pm</v>
+        <v>7/5/2026, 12:06:05 am</v>
       </c>
       <c r="E32" t="str">
         <v>Success</v>
@@ -952,13 +952,13 @@
         <v>https://www.softwebsolutions.com/finance-industry/</v>
       </c>
       <c r="B33">
-        <v>6.5</v>
+        <v>6.37</v>
       </c>
       <c r="C33" t="str">
-        <v>5/5/2026, 3:27:36 pm</v>
+        <v>7/5/2026, 12:06:11 am</v>
       </c>
       <c r="D33" t="str">
-        <v>5/5/2026, 3:27:43 pm</v>
+        <v>7/5/2026, 12:06:17 am</v>
       </c>
       <c r="E33" t="str">
         <v>Success</v>
@@ -969,13 +969,13 @@
         <v>https://www.softwebsolutions.com/flutter-app-development-services/</v>
       </c>
       <c r="B34">
-        <v>1.11</v>
+        <v>9.8</v>
       </c>
       <c r="C34" t="str">
-        <v>5/5/2026, 3:27:50 pm</v>
+        <v>7/5/2026, 12:06:22 am</v>
       </c>
       <c r="D34" t="str">
-        <v>5/5/2026, 3:27:51 pm</v>
+        <v>7/5/2026, 12:06:32 am</v>
       </c>
       <c r="E34" t="str">
         <v>Success</v>
@@ -986,13 +986,13 @@
         <v>https://www.softwebsolutions.com/front-end-development/</v>
       </c>
       <c r="B35">
-        <v>4.53</v>
+        <v>8.39</v>
       </c>
       <c r="C35" t="str">
-        <v>5/5/2026, 3:27:58 pm</v>
+        <v>7/5/2026, 12:06:35 am</v>
       </c>
       <c r="D35" t="str">
-        <v>5/5/2026, 3:28:02 pm</v>
+        <v>7/5/2026, 12:06:44 am</v>
       </c>
       <c r="E35" t="str">
         <v>Success</v>
@@ -1003,13 +1003,13 @@
         <v>https://www.softwebsolutions.com/full-stack-development-company/</v>
       </c>
       <c r="B36">
-        <v>1.47</v>
+        <v>6.66</v>
       </c>
       <c r="C36" t="str">
-        <v>5/5/2026, 3:28:10 pm</v>
+        <v>7/5/2026, 12:06:52 am</v>
       </c>
       <c r="D36" t="str">
-        <v>5/5/2026, 3:28:12 pm</v>
+        <v>7/5/2026, 12:06:59 am</v>
       </c>
       <c r="E36" t="str">
         <v>Success</v>
@@ -1020,13 +1020,13 @@
         <v>https://www.softwebsolutions.com/generative-ai-consulting-services/</v>
       </c>
       <c r="B37">
-        <v>5.85</v>
+        <v>5.87</v>
       </c>
       <c r="C37" t="str">
-        <v>5/5/2026, 3:28:20 pm</v>
+        <v>7/5/2026, 12:07:06 am</v>
       </c>
       <c r="D37" t="str">
-        <v>5/5/2026, 3:28:26 pm</v>
+        <v>7/5/2026, 12:07:12 am</v>
       </c>
       <c r="E37" t="str">
         <v>Success</v>
@@ -1037,13 +1037,13 @@
         <v>https://www.softwebsolutions.com/hybrid-cloud-services/</v>
       </c>
       <c r="B38">
-        <v>4.99</v>
+        <v>2.06</v>
       </c>
       <c r="C38" t="str">
-        <v>5/5/2026, 3:28:32 pm</v>
+        <v>7/5/2026, 12:07:18 am</v>
       </c>
       <c r="D38" t="str">
-        <v>5/5/2026, 3:28:37 pm</v>
+        <v>7/5/2026, 12:07:20 am</v>
       </c>
       <c r="E38" t="str">
         <v>Success</v>
@@ -1054,13 +1054,13 @@
         <v>https://www.softwebsolutions.com/image-annotation-services/</v>
       </c>
       <c r="B39">
-        <v>1.83</v>
+        <v>1.56</v>
       </c>
       <c r="C39" t="str">
-        <v>5/5/2026, 3:28:42 pm</v>
+        <v>7/5/2026, 12:07:24 am</v>
       </c>
       <c r="D39" t="str">
-        <v>5/5/2026, 3:28:44 pm</v>
+        <v>7/5/2026, 12:07:26 am</v>
       </c>
       <c r="E39" t="str">
         <v>Success</v>
@@ -1068,16 +1068,16 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>https://www.softwebsolutions.com/image-processing-services/</v>
+        <v>https://www.softwebsolutions.com/production-line-monitoring-solution/</v>
       </c>
       <c r="B40">
-        <v>8.04</v>
+        <v>5.69</v>
       </c>
       <c r="C40" t="str">
-        <v>5/5/2026, 3:22:34 pm</v>
+        <v>7/5/2026, 12:00:43 am</v>
       </c>
       <c r="D40" t="str">
-        <v>5/5/2026, 3:22:42 pm</v>
+        <v>7/5/2026, 12:00:49 am</v>
       </c>
       <c r="E40" t="str">
         <v>Success</v>
@@ -1085,16 +1085,16 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>https://www.softwebsolutions.com/industries/</v>
+        <v>https://www.softwebsolutions.com/python-development-services/</v>
       </c>
       <c r="B41">
-        <v>1.84</v>
+        <v>6.84</v>
       </c>
       <c r="C41" t="str">
-        <v>5/5/2026, 3:22:48 pm</v>
+        <v>7/5/2026, 12:00:56 am</v>
       </c>
       <c r="D41" t="str">
-        <v>5/5/2026, 3:22:49 pm</v>
+        <v>7/5/2026, 12:01:02 am</v>
       </c>
       <c r="E41" t="str">
         <v>Success</v>
@@ -1102,16 +1102,16 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>https://www.softwebsolutions.com/intelligent-automation-services/</v>
+        <v>https://www.softwebsolutions.com/quality-inspection-in-manufacturing/</v>
       </c>
       <c r="B42">
-        <v>1.27</v>
+        <v>5.2</v>
       </c>
       <c r="C42" t="str">
-        <v>5/5/2026, 3:22:53 pm</v>
+        <v>7/5/2026, 12:01:10 am</v>
       </c>
       <c r="D42" t="str">
-        <v>5/5/2026, 3:22:54 pm</v>
+        <v>7/5/2026, 12:01:15 am</v>
       </c>
       <c r="E42" t="str">
         <v>Success</v>
@@ -1119,16 +1119,16 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>https://www.softwebsolutions.com/intelligent-document-processing-solutions/</v>
+        <v>https://www.softwebsolutions.com/rag-as-a-service/</v>
       </c>
       <c r="B43">
-        <v>4.93</v>
+        <v>1.2</v>
       </c>
       <c r="C43" t="str">
-        <v>5/5/2026, 3:22:59 pm</v>
+        <v>7/5/2026, 12:01:22 am</v>
       </c>
       <c r="D43" t="str">
-        <v>5/5/2026, 3:23:04 pm</v>
+        <v>7/5/2026, 12:01:23 am</v>
       </c>
       <c r="E43" t="str">
         <v>Success</v>
@@ -1136,16 +1136,16 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>https://www.softwebsolutions.com/intelligent-forecasting-services/</v>
+        <v>https://www.softwebsolutions.com/react-native-app-development-services/</v>
       </c>
       <c r="B44">
-        <v>6.23</v>
+        <v>5.58</v>
       </c>
       <c r="C44" t="str">
-        <v>5/5/2026, 3:23:09 pm</v>
+        <v>7/5/2026, 12:01:30 am</v>
       </c>
       <c r="D44" t="str">
-        <v>5/5/2026, 3:23:16 pm</v>
+        <v>7/5/2026, 12:01:36 am</v>
       </c>
       <c r="E44" t="str">
         <v>Success</v>
@@ -1153,16 +1153,16 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>https://www.softwebsolutions.com/intelligent-video-analytics-solutions/</v>
+        <v>https://www.softwebsolutions.com/reactjs-development-services/</v>
       </c>
       <c r="B45">
-        <v>0.97</v>
+        <v>4.84</v>
       </c>
       <c r="C45" t="str">
-        <v>5/5/2026, 3:23:22 pm</v>
+        <v>7/5/2026, 12:01:42 am</v>
       </c>
       <c r="D45" t="str">
-        <v>5/5/2026, 3:23:23 pm</v>
+        <v>7/5/2026, 12:01:47 am</v>
       </c>
       <c r="E45" t="str">
         <v>Success</v>
@@ -1170,16 +1170,16 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>https://www.softwebsolutions.com/intelligent-virtual-assistant/</v>
+        <v>https://www.softwebsolutions.com/recommendation-system-development-services/</v>
       </c>
       <c r="B46">
-        <v>1.33</v>
+        <v>4.84</v>
       </c>
       <c r="C46" t="str">
-        <v>5/5/2026, 3:23:28 pm</v>
+        <v>7/5/2026, 12:01:53 am</v>
       </c>
       <c r="D46" t="str">
-        <v>5/5/2026, 3:23:29 pm</v>
+        <v>7/5/2026, 12:01:58 am</v>
       </c>
       <c r="E46" t="str">
         <v>Success</v>
@@ -1187,16 +1187,16 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>https://www.softwebsolutions.com/inventory-analytics-dashboards/</v>
+        <v>https://www.softwebsolutions.com/salesforce-ai-consulting/</v>
       </c>
       <c r="B47">
-        <v>1.08</v>
+        <v>5.08</v>
       </c>
       <c r="C47" t="str">
-        <v>5/5/2026, 3:23:36 pm</v>
+        <v>7/5/2026, 12:02:04 am</v>
       </c>
       <c r="D47" t="str">
-        <v>5/5/2026, 3:23:37 pm</v>
+        <v>7/5/2026, 12:02:09 am</v>
       </c>
       <c r="E47" t="str">
         <v>Success</v>
@@ -1204,16 +1204,16 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>https://www.softwebsolutions.com/large-language-model-development/</v>
+        <v>https://www.softwebsolutions.com/salesforce-cloud-services/</v>
       </c>
       <c r="B48">
-        <v>7.36</v>
+        <v>5.11</v>
       </c>
       <c r="C48" t="str">
-        <v>5/5/2026, 3:23:44 pm</v>
+        <v>7/5/2026, 12:02:16 am</v>
       </c>
       <c r="D48" t="str">
-        <v>5/5/2026, 3:23:51 pm</v>
+        <v>7/5/2026, 12:02:21 am</v>
       </c>
       <c r="E48" t="str">
         <v>Success</v>
@@ -1221,16 +1221,16 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>https://www.softwebsolutions.com/legacy-application-modernization/</v>
+        <v>https://www.softwebsolutions.com/salesforce-commerce-cloud-services/</v>
       </c>
       <c r="B49">
-        <v>5.21</v>
+        <v>5.74</v>
       </c>
       <c r="C49" t="str">
-        <v>5/5/2026, 3:23:58 pm</v>
+        <v>7/5/2026, 12:02:28 am</v>
       </c>
       <c r="D49" t="str">
-        <v>5/5/2026, 3:24:03 pm</v>
+        <v>7/5/2026, 12:02:34 am</v>
       </c>
       <c r="E49" t="str">
         <v>Success</v>
@@ -1238,16 +1238,16 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>https://www.softwebsolutions.com/llmops-services/</v>
+        <v>https://www.softwebsolutions.com/salesforce-consulting-services/</v>
       </c>
       <c r="B50">
-        <v>1.01</v>
+        <v>4.78</v>
       </c>
       <c r="C50" t="str">
-        <v>5/5/2026, 3:24:10 pm</v>
+        <v>7/5/2026, 12:02:42 am</v>
       </c>
       <c r="D50" t="str">
-        <v>5/5/2026, 3:24:11 pm</v>
+        <v>7/5/2026, 12:02:47 am</v>
       </c>
       <c r="E50" t="str">
         <v>Success</v>
@@ -1255,16 +1255,16 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>https://www.softwebsolutions.com/machine-learning-consulting/</v>
+        <v>https://www.softwebsolutions.com/salesforce-data-cloud-services/</v>
       </c>
       <c r="B51">
-        <v>5.65</v>
+        <v>5.3</v>
       </c>
       <c r="C51" t="str">
-        <v>5/5/2026, 3:24:18 pm</v>
+        <v>7/5/2026, 12:02:53 am</v>
       </c>
       <c r="D51" t="str">
-        <v>5/5/2026, 3:24:24 pm</v>
+        <v>7/5/2026, 12:02:59 am</v>
       </c>
       <c r="E51" t="str">
         <v>Success</v>
@@ -1272,16 +1272,16 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>https://www.softwebsolutions.com/machine-learning-services/</v>
+        <v>https://www.softwebsolutions.com/salesforce-development-services/</v>
       </c>
       <c r="B52">
-        <v>1.95</v>
+        <v>8.45</v>
       </c>
       <c r="C52" t="str">
-        <v>5/5/2026, 3:24:31 pm</v>
+        <v>7/5/2026, 12:03:06 am</v>
       </c>
       <c r="D52" t="str">
-        <v>5/5/2026, 3:24:33 pm</v>
+        <v>7/5/2026, 12:03:14 am</v>
       </c>
       <c r="E52" t="str">
         <v>Success</v>
@@ -1289,16 +1289,16 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>https://www.softwebsolutions.com/machine-monitoring-system/</v>
+        <v>https://www.softwebsolutions.com/salesforce-experience-cloud-services/</v>
       </c>
       <c r="B53">
-        <v>5.43</v>
+        <v>1.5</v>
       </c>
       <c r="C53" t="str">
-        <v>5/5/2026, 3:24:39 pm</v>
+        <v>7/5/2026, 12:03:18 am</v>
       </c>
       <c r="D53" t="str">
-        <v>5/5/2026, 3:24:44 pm</v>
+        <v>7/5/2026, 12:03:20 am</v>
       </c>
       <c r="E53" t="str">
         <v>Success</v>
@@ -1306,16 +1306,16 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>https://www.softwebsolutions.com/managed-services-provider/</v>
+        <v>https://www.softwebsolutions.com/salesforce-implementation-services/</v>
       </c>
       <c r="B54">
-        <v>1.53</v>
+        <v>8.8</v>
       </c>
       <c r="C54" t="str">
-        <v>5/5/2026, 3:24:51 pm</v>
+        <v>7/5/2026, 12:03:26 am</v>
       </c>
       <c r="D54" t="str">
-        <v>5/5/2026, 3:24:53 pm</v>
+        <v>7/5/2026, 12:03:34 am</v>
       </c>
       <c r="E54" t="str">
         <v>Success</v>
@@ -1323,16 +1323,16 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>https://www.softwebsolutions.com/manufacturing-industry/</v>
+        <v>https://www.softwebsolutions.com/salesforce-integration-services/</v>
       </c>
       <c r="B55">
-        <v>1.6</v>
+        <v>4.96</v>
       </c>
       <c r="C55" t="str">
-        <v>5/5/2026, 3:25:01 pm</v>
+        <v>7/5/2026, 12:03:41 am</v>
       </c>
       <c r="D55" t="str">
-        <v>5/5/2026, 3:25:03 pm</v>
+        <v>7/5/2026, 12:03:46 am</v>
       </c>
       <c r="E55" t="str">
         <v>Success</v>
@@ -1340,16 +1340,16 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>https://www.softwebsolutions.com/microservices/</v>
+        <v>https://www.softwebsolutions.com/salesforce-migration-services/</v>
       </c>
       <c r="B56">
-        <v>6.34</v>
+        <v>5.57</v>
       </c>
       <c r="C56" t="str">
-        <v>5/5/2026, 3:25:09 pm</v>
+        <v>7/5/2026, 12:03:52 am</v>
       </c>
       <c r="D56" t="str">
-        <v>5/5/2026, 3:25:16 pm</v>
+        <v>7/5/2026, 12:03:57 am</v>
       </c>
       <c r="E56" t="str">
         <v>Success</v>
@@ -1357,16 +1357,16 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>https://www.softwebsolutions.com/microsoft-365-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/salesforce-revenue-cloud-advanced/</v>
       </c>
       <c r="B57">
-        <v>1.37</v>
+        <v>6.44</v>
       </c>
       <c r="C57" t="str">
-        <v>5/5/2026, 3:25:23 pm</v>
+        <v>7/5/2026, 12:04:05 am</v>
       </c>
       <c r="D57" t="str">
-        <v>5/5/2026, 3:25:24 pm</v>
+        <v>7/5/2026, 12:04:11 am</v>
       </c>
       <c r="E57" t="str">
         <v>Success</v>
@@ -1374,16 +1374,16 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>https://www.softwebsolutions.com/microsoft-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/salesforce-revenue-cloud-services/</v>
       </c>
       <c r="B58">
-        <v>5.99</v>
+        <v>5.19</v>
       </c>
       <c r="C58" t="str">
-        <v>5/5/2026, 3:25:30 pm</v>
+        <v>7/5/2026, 12:04:18 am</v>
       </c>
       <c r="D58" t="str">
-        <v>5/5/2026, 3:25:36 pm</v>
+        <v>7/5/2026, 12:04:23 am</v>
       </c>
       <c r="E58" t="str">
         <v>Success</v>
@@ -1391,16 +1391,16 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>https://www.softwebsolutions.com/microsoft-copilot-studio-consulting/</v>
+        <v>https://www.softwebsolutions.com/salesforce-sales-cloud-services/</v>
       </c>
       <c r="B59">
-        <v>1.12</v>
+        <v>0.95</v>
       </c>
       <c r="C59" t="str">
-        <v>5/5/2026, 3:25:43 pm</v>
+        <v>7/5/2026, 12:04:29 am</v>
       </c>
       <c r="D59" t="str">
-        <v>5/5/2026, 3:25:44 pm</v>
+        <v>7/5/2026, 12:04:30 am</v>
       </c>
       <c r="E59" t="str">
         <v>Success</v>
@@ -1408,16 +1408,16 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>https://www.softwebsolutions.com/microsoft-hololens-app-development-company/</v>
+        <v>https://www.softwebsolutions.com/semiconductor/</v>
       </c>
       <c r="B60">
-        <v>1.07</v>
+        <v>1.21</v>
       </c>
       <c r="C60" t="str">
-        <v>5/5/2026, 3:25:51 pm</v>
+        <v>7/5/2026, 12:04:38 am</v>
       </c>
       <c r="D60" t="str">
-        <v>5/5/2026, 3:25:52 pm</v>
+        <v>7/5/2026, 12:04:39 am</v>
       </c>
       <c r="E60" t="str">
         <v>Success</v>
@@ -1425,16 +1425,16 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>https://www.softwebsolutions.com/microsoft-viva-consulting/</v>
+        <v>https://www.softwebsolutions.com/sharepoint-consulting-services/</v>
       </c>
       <c r="B61">
-        <v>4.09</v>
+        <v>1.09</v>
       </c>
       <c r="C61" t="str">
-        <v>5/5/2026, 3:25:58 pm</v>
+        <v>7/5/2026, 12:04:46 am</v>
       </c>
       <c r="D61" t="str">
-        <v>5/5/2026, 3:26:02 pm</v>
+        <v>7/5/2026, 12:04:47 am</v>
       </c>
       <c r="E61" t="str">
         <v>Success</v>
@@ -1442,16 +1442,16 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>https://www.softwebsolutions.com/mlops-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/simple-reflex-ai-agents/</v>
       </c>
       <c r="B62">
-        <v>1.5</v>
+        <v>1.11</v>
       </c>
       <c r="C62" t="str">
-        <v>5/5/2026, 3:26:09 pm</v>
+        <v>7/5/2026, 12:04:55 am</v>
       </c>
       <c r="D62" t="str">
-        <v>5/5/2026, 3:26:11 pm</v>
+        <v>7/5/2026, 12:04:56 am</v>
       </c>
       <c r="E62" t="str">
         <v>Success</v>
@@ -1459,16 +1459,16 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>https://www.softwebsolutions.com/mobile-app-development/</v>
+        <v>https://www.softwebsolutions.com/sitecore-implementation/</v>
       </c>
       <c r="B63">
-        <v>7.88</v>
+        <v>1.45</v>
       </c>
       <c r="C63" t="str">
-        <v>5/5/2026, 3:26:17 pm</v>
+        <v>7/5/2026, 12:05:04 am</v>
       </c>
       <c r="D63" t="str">
-        <v>5/5/2026, 3:26:25 pm</v>
+        <v>7/5/2026, 12:05:05 am</v>
       </c>
       <c r="E63" t="str">
         <v>Success</v>
@@ -1476,16 +1476,16 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>https://www.softwebsolutions.com/mulesoft-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/sitecore-managed-services/</v>
       </c>
       <c r="B64">
-        <v>4.98</v>
+        <v>1.81</v>
       </c>
       <c r="C64" t="str">
-        <v>5/5/2026, 3:26:30 pm</v>
+        <v>7/5/2026, 12:05:11 am</v>
       </c>
       <c r="D64" t="str">
-        <v>5/5/2026, 3:26:35 pm</v>
+        <v>7/5/2026, 12:05:13 am</v>
       </c>
       <c r="E64" t="str">
         <v>Success</v>
@@ -1493,16 +1493,16 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>https://www.softwebsolutions.com/multicloud-managed-services/</v>
+        <v>https://www.softwebsolutions.com/snowflake-consulting-services/</v>
       </c>
       <c r="B65">
-        <v>1.15</v>
+        <v>5.92</v>
       </c>
       <c r="C65" t="str">
-        <v>5/5/2026, 3:26:42 pm</v>
+        <v>7/5/2026, 12:05:19 am</v>
       </c>
       <c r="D65" t="str">
-        <v>5/5/2026, 3:26:44 pm</v>
+        <v>7/5/2026, 12:05:25 am</v>
       </c>
       <c r="E65" t="str">
         <v>Success</v>
@@ -1510,16 +1510,16 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>https://www.softwebsolutions.com/natural-language-processing-services/</v>
+        <v>https://www.softwebsolutions.com/solutions/</v>
       </c>
       <c r="B66">
-        <v>7.07</v>
+        <v>1.07</v>
       </c>
       <c r="C66" t="str">
-        <v>5/5/2026, 3:26:49 pm</v>
+        <v>7/5/2026, 12:05:31 am</v>
       </c>
       <c r="D66" t="str">
-        <v>5/5/2026, 3:26:56 pm</v>
+        <v>7/5/2026, 12:05:32 am</v>
       </c>
       <c r="E66" t="str">
         <v>Success</v>
@@ -1527,16 +1527,16 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>https://www.softwebsolutions.com/net-maui-development-services/</v>
+        <v>https://www.softwebsolutions.com/supply-chain-automation-solution/</v>
       </c>
       <c r="B67">
-        <v>1.06</v>
+        <v>0.95</v>
       </c>
       <c r="C67" t="str">
-        <v>5/5/2026, 3:27:03 pm</v>
+        <v>7/5/2026, 12:05:38 am</v>
       </c>
       <c r="D67" t="str">
-        <v>5/5/2026, 3:27:04 pm</v>
+        <v>7/5/2026, 12:05:39 am</v>
       </c>
       <c r="E67" t="str">
         <v>Success</v>
@@ -1544,16 +1544,16 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>https://www.softwebsolutions.com/nodejs-application-development/</v>
+        <v>https://www.softwebsolutions.com/supply-chain-bot-development/</v>
       </c>
       <c r="B68">
-        <v>0.95</v>
+        <v>1.61</v>
       </c>
       <c r="C68" t="str">
-        <v>5/5/2026, 3:27:10 pm</v>
+        <v>7/5/2026, 12:05:45 am</v>
       </c>
       <c r="D68" t="str">
-        <v>5/5/2026, 3:27:11 pm</v>
+        <v>7/5/2026, 12:05:47 am</v>
       </c>
       <c r="E68" t="str">
         <v>Success</v>
@@ -1561,16 +1561,16 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>https://www.softwebsolutions.com/partner-relationship-management/</v>
+        <v>https://www.softwebsolutions.com/supply-chain/</v>
       </c>
       <c r="B69">
-        <v>1.03</v>
+        <v>7.21</v>
       </c>
       <c r="C69" t="str">
-        <v>5/5/2026, 3:27:17 pm</v>
+        <v>7/5/2026, 12:05:50 am</v>
       </c>
       <c r="D69" t="str">
-        <v>5/5/2026, 3:27:18 pm</v>
+        <v>7/5/2026, 12:05:57 am</v>
       </c>
       <c r="E69" t="str">
         <v>Success</v>
@@ -1578,16 +1578,16 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>https://www.softwebsolutions.com/power-automate-consulting/</v>
+        <v>https://www.softwebsolutions.com/surface-defect-detection/</v>
       </c>
       <c r="B70">
-        <v>1.08</v>
+        <v>6.67</v>
       </c>
       <c r="C70" t="str">
-        <v>5/5/2026, 3:27:25 pm</v>
+        <v>7/5/2026, 12:06:02 am</v>
       </c>
       <c r="D70" t="str">
-        <v>5/5/2026, 3:27:26 pm</v>
+        <v>7/5/2026, 12:06:09 am</v>
       </c>
       <c r="E70" t="str">
         <v>Success</v>
@@ -1595,16 +1595,16 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>https://www.softwebsolutions.com/power-bi-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/tableau-consulting-services/</v>
       </c>
       <c r="B71">
-        <v>4.68</v>
+        <v>4.72</v>
       </c>
       <c r="C71" t="str">
-        <v>5/5/2026, 3:27:33 pm</v>
+        <v>7/5/2026, 12:06:15 am</v>
       </c>
       <c r="D71" t="str">
-        <v>5/5/2026, 3:27:38 pm</v>
+        <v>7/5/2026, 12:06:19 am</v>
       </c>
       <c r="E71" t="str">
         <v>Success</v>
@@ -1612,16 +1612,16 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>https://www.softwebsolutions.com/power-bi-oee-dashboards/</v>
+        <v>https://www.softwebsolutions.com/vision-based-eol-detection/</v>
       </c>
       <c r="B72">
-        <v>1.18</v>
+        <v>14.25</v>
       </c>
       <c r="C72" t="str">
-        <v>5/5/2026, 3:27:45 pm</v>
+        <v>7/5/2026, 12:06:24 am</v>
       </c>
       <c r="D72" t="str">
-        <v>5/5/2026, 3:27:46 pm</v>
+        <v>7/5/2026, 12:06:38 am</v>
       </c>
       <c r="E72" t="str">
         <v>Success</v>
@@ -1629,16 +1629,16 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>https://www.softwebsolutions.com/power-platform-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/wafer-defect-detection/</v>
       </c>
       <c r="B73">
-        <v>1.26</v>
+        <v>4.91</v>
       </c>
       <c r="C73" t="str">
-        <v>5/5/2026, 3:27:52 pm</v>
+        <v>7/5/2026, 12:06:43 am</v>
       </c>
       <c r="D73" t="str">
-        <v>5/5/2026, 3:27:53 pm</v>
+        <v>7/5/2026, 12:06:48 am</v>
       </c>
       <c r="E73" t="str">
         <v>Success</v>
@@ -1646,16 +1646,16 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>https://www.softwebsolutions.com/powerapps-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/web-application-development/</v>
       </c>
       <c r="B74">
-        <v>1.36</v>
+        <v>2.29</v>
       </c>
       <c r="C74" t="str">
-        <v>5/5/2026, 3:27:59 pm</v>
+        <v>7/5/2026, 12:06:55 am</v>
       </c>
       <c r="D74" t="str">
-        <v>5/5/2026, 3:28:00 pm</v>
+        <v>7/5/2026, 12:06:57 am</v>
       </c>
       <c r="E74" t="str">
         <v>Success</v>
@@ -1663,16 +1663,16 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>https://www.softwebsolutions.com/predictive-analytics-services/</v>
+        <v>https://www.softwebsolutions.com/wordpress-development-services/</v>
       </c>
       <c r="B75">
-        <v>5.23</v>
+        <v>2.17</v>
       </c>
       <c r="C75" t="str">
-        <v>5/5/2026, 3:28:06 pm</v>
+        <v>7/5/2026, 12:07:06 am</v>
       </c>
       <c r="D75" t="str">
-        <v>5/5/2026, 3:28:12 pm</v>
+        <v>7/5/2026, 12:07:08 am</v>
       </c>
       <c r="E75" t="str">
         <v>Success</v>
@@ -1680,16 +1680,16 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>https://www.softwebsolutions.com/product-engineering-service/</v>
+        <v>https://www.softwebsolutions.com/image-processing-services/</v>
       </c>
       <c r="B76">
-        <v>5.75</v>
+        <v>6.01</v>
       </c>
       <c r="C76" t="str">
-        <v>5/5/2026, 3:28:20 pm</v>
+        <v>7/5/2026, 12:00:43 am</v>
       </c>
       <c r="D76" t="str">
-        <v>5/5/2026, 3:28:26 pm</v>
+        <v>7/5/2026, 12:00:49 am</v>
       </c>
       <c r="E76" t="str">
         <v>Success</v>
@@ -1697,16 +1697,16 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>https://www.softwebsolutions.com/product-information-management-system/</v>
+        <v>https://www.softwebsolutions.com/industries/</v>
       </c>
       <c r="B77">
-        <v>6</v>
+        <v>6.02</v>
       </c>
       <c r="C77" t="str">
-        <v>5/5/2026, 3:28:32 pm</v>
+        <v>7/5/2026, 12:00:56 am</v>
       </c>
       <c r="D77" t="str">
-        <v>5/5/2026, 3:28:38 pm</v>
+        <v>7/5/2026, 12:01:02 am</v>
       </c>
       <c r="E77" t="str">
         <v>Success</v>
@@ -1714,16 +1714,16 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>https://www.softwebsolutions.com/</v>
+        <v>https://www.softwebsolutions.com/intelligent-automation-services/</v>
       </c>
       <c r="B78">
-        <v>7.79</v>
+        <v>1.57</v>
       </c>
       <c r="C78" t="str">
-        <v>5/5/2026, 3:22:35 pm</v>
+        <v>7/5/2026, 12:01:09 am</v>
       </c>
       <c r="D78" t="str">
-        <v>5/5/2026, 3:22:43 pm</v>
+        <v>7/5/2026, 12:01:11 am</v>
       </c>
       <c r="E78" t="str">
         <v>Success</v>
@@ -1731,16 +1731,16 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>https://www.softwebsolutions.com/about-softweb-solutions/</v>
+        <v>https://www.softwebsolutions.com/intelligent-document-processing-solutions/</v>
       </c>
       <c r="B79">
-        <v>4.46</v>
+        <v>1.46</v>
       </c>
       <c r="C79" t="str">
-        <v>5/5/2026, 3:22:48 pm</v>
+        <v>7/5/2026, 12:01:19 am</v>
       </c>
       <c r="D79" t="str">
-        <v>5/5/2026, 3:22:52 pm</v>
+        <v>7/5/2026, 12:01:21 am</v>
       </c>
       <c r="E79" t="str">
         <v>Success</v>
@@ -1748,16 +1748,16 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>https://www.softwebsolutions.com/adaptive-ai-development-company/</v>
+        <v>https://www.softwebsolutions.com/intelligent-forecasting-services/</v>
       </c>
       <c r="B80">
-        <v>4.59</v>
+        <v>4.99</v>
       </c>
       <c r="C80" t="str">
-        <v>5/5/2026, 3:22:58 pm</v>
+        <v>7/5/2026, 12:01:28 am</v>
       </c>
       <c r="D80" t="str">
-        <v>5/5/2026, 3:23:02 pm</v>
+        <v>7/5/2026, 12:01:33 am</v>
       </c>
       <c r="E80" t="str">
         <v>Success</v>
@@ -1765,16 +1765,16 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>https://www.softwebsolutions.com/agentforce-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/intelligent-video-analytics-solutions/</v>
       </c>
       <c r="B81">
-        <v>1.44</v>
+        <v>0.99</v>
       </c>
       <c r="C81" t="str">
-        <v>5/5/2026, 3:23:08 pm</v>
+        <v>7/5/2026, 12:01:40 am</v>
       </c>
       <c r="D81" t="str">
-        <v>5/5/2026, 3:23:10 pm</v>
+        <v>7/5/2026, 12:01:41 am</v>
       </c>
       <c r="E81" t="str">
         <v>Success</v>
@@ -1782,16 +1782,16 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>https://www.softwebsolutions.com/agentic-ai-services/</v>
+        <v>https://www.softwebsolutions.com/intelligent-virtual-assistant/</v>
       </c>
       <c r="B82">
-        <v>4.99</v>
+        <v>4.91</v>
       </c>
       <c r="C82" t="str">
-        <v>5/5/2026, 3:23:16 pm</v>
+        <v>7/5/2026, 12:01:50 am</v>
       </c>
       <c r="D82" t="str">
-        <v>5/5/2026, 3:23:21 pm</v>
+        <v>7/5/2026, 12:01:55 am</v>
       </c>
       <c r="E82" t="str">
         <v>Success</v>
@@ -1799,16 +1799,16 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>https://www.softwebsolutions.com/ai-agent-development-company/</v>
+        <v>https://www.softwebsolutions.com/inventory-analytics-dashboards/</v>
       </c>
       <c r="B83">
-        <v>5.21</v>
+        <v>1.5</v>
       </c>
       <c r="C83" t="str">
-        <v>5/5/2026, 3:23:27 pm</v>
+        <v>7/5/2026, 12:02:02 am</v>
       </c>
       <c r="D83" t="str">
-        <v>5/5/2026, 3:23:32 pm</v>
+        <v>7/5/2026, 12:02:04 am</v>
       </c>
       <c r="E83" t="str">
         <v>Success</v>
@@ -1816,16 +1816,16 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>https://www.softwebsolutions.com/ai-anomaly-detection/</v>
+        <v>https://www.softwebsolutions.com/large-language-model-development/</v>
       </c>
       <c r="B84">
-        <v>0.95</v>
+        <v>5.97</v>
       </c>
       <c r="C84" t="str">
-        <v>5/5/2026, 3:23:37 pm</v>
+        <v>7/5/2026, 12:02:09 am</v>
       </c>
       <c r="D84" t="str">
-        <v>5/5/2026, 3:23:38 pm</v>
+        <v>7/5/2026, 12:02:15 am</v>
       </c>
       <c r="E84" t="str">
         <v>Success</v>
@@ -1833,16 +1833,16 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>https://www.softwebsolutions.com/ai-automation-testing-services/</v>
+        <v>https://www.softwebsolutions.com/legacy-application-modernization/</v>
       </c>
       <c r="B85">
-        <v>1.27</v>
+        <v>1.21</v>
       </c>
       <c r="C85" t="str">
-        <v>5/5/2026, 3:23:45 pm</v>
+        <v>7/5/2026, 12:02:22 am</v>
       </c>
       <c r="D85" t="str">
-        <v>5/5/2026, 3:23:47 pm</v>
+        <v>7/5/2026, 12:02:24 am</v>
       </c>
       <c r="E85" t="str">
         <v>Success</v>
@@ -1850,16 +1850,16 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>https://www.softwebsolutions.com/ai-chatbot-development-company/</v>
+        <v>https://www.softwebsolutions.com/llmops-services/</v>
       </c>
       <c r="B86">
-        <v>1.26</v>
+        <v>1.2</v>
       </c>
       <c r="C86" t="str">
-        <v>5/5/2026, 3:23:53 pm</v>
+        <v>7/5/2026, 12:02:30 am</v>
       </c>
       <c r="D86" t="str">
-        <v>5/5/2026, 3:23:54 pm</v>
+        <v>7/5/2026, 12:02:31 am</v>
       </c>
       <c r="E86" t="str">
         <v>Success</v>
@@ -1867,16 +1867,16 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>https://www.softwebsolutions.com/ai-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/machine-learning-consulting/</v>
       </c>
       <c r="B87">
-        <v>5.34</v>
+        <v>1.53</v>
       </c>
       <c r="C87" t="str">
-        <v>5/5/2026, 3:24:00 pm</v>
+        <v>7/5/2026, 12:02:39 am</v>
       </c>
       <c r="D87" t="str">
-        <v>5/5/2026, 3:24:05 pm</v>
+        <v>7/5/2026, 12:02:40 am</v>
       </c>
       <c r="E87" t="str">
         <v>Success</v>
@@ -1884,16 +1884,16 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>https://www.softwebsolutions.com/ai-defect-detection-visual-inspection/</v>
+        <v>https://www.softwebsolutions.com/machine-learning-services/</v>
       </c>
       <c r="B88">
-        <v>1.21</v>
+        <v>1.34</v>
       </c>
       <c r="C88" t="str">
-        <v>5/5/2026, 3:24:11 pm</v>
+        <v>7/5/2026, 12:02:48 am</v>
       </c>
       <c r="D88" t="str">
-        <v>5/5/2026, 3:24:12 pm</v>
+        <v>7/5/2026, 12:02:49 am</v>
       </c>
       <c r="E88" t="str">
         <v>Success</v>
@@ -1901,16 +1901,16 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>https://www.softwebsolutions.com/ai-development-services/</v>
+        <v>https://www.softwebsolutions.com/machine-monitoring-system/</v>
       </c>
       <c r="B89">
-        <v>1.67</v>
+        <v>5.09</v>
       </c>
       <c r="C89" t="str">
-        <v>5/5/2026, 3:24:19 pm</v>
+        <v>7/5/2026, 12:02:57 am</v>
       </c>
       <c r="D89" t="str">
-        <v>5/5/2026, 3:24:21 pm</v>
+        <v>7/5/2026, 12:03:02 am</v>
       </c>
       <c r="E89" t="str">
         <v>Success</v>
@@ -1918,16 +1918,16 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>https://www.softwebsolutions.com/ai-powered-inventory-management/</v>
+        <v>https://www.softwebsolutions.com/managed-services-provider/</v>
       </c>
       <c r="B90">
-        <v>1.25</v>
+        <v>5.97</v>
       </c>
       <c r="C90" t="str">
-        <v>5/5/2026, 3:24:26 pm</v>
+        <v>7/5/2026, 12:03:09 am</v>
       </c>
       <c r="D90" t="str">
-        <v>5/5/2026, 3:24:27 pm</v>
+        <v>7/5/2026, 12:03:15 am</v>
       </c>
       <c r="E90" t="str">
         <v>Success</v>
@@ -1935,16 +1935,16 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>https://www.softwebsolutions.com/ai-prompt-engineering-services/</v>
+        <v>https://www.softwebsolutions.com/manufacturing-industry/</v>
       </c>
       <c r="B91">
-        <v>7.05</v>
+        <v>1.59</v>
       </c>
       <c r="C91" t="str">
-        <v>5/5/2026, 3:24:34 pm</v>
+        <v>7/5/2026, 12:03:20 am</v>
       </c>
       <c r="D91" t="str">
-        <v>5/5/2026, 3:24:42 pm</v>
+        <v>7/5/2026, 12:03:21 am</v>
       </c>
       <c r="E91" t="str">
         <v>Success</v>
@@ -1952,16 +1952,16 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>https://www.softwebsolutions.com/aiops-solutions/</v>
+        <v>https://www.softwebsolutions.com/microservices/</v>
       </c>
       <c r="B92">
-        <v>1.23</v>
+        <v>9.09</v>
       </c>
       <c r="C92" t="str">
-        <v>5/5/2026, 3:24:50 pm</v>
+        <v>7/5/2026, 12:03:27 am</v>
       </c>
       <c r="D92" t="str">
-        <v>5/5/2026, 3:24:52 pm</v>
+        <v>7/5/2026, 12:03:36 am</v>
       </c>
       <c r="E92" t="str">
         <v>Success</v>
@@ -1969,16 +1969,16 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>https://www.softwebsolutions.com/application-managed-services/</v>
+        <v>https://www.softwebsolutions.com/microsoft-365-consulting-services/</v>
       </c>
       <c r="B93">
-        <v>4.28</v>
+        <v>1.69</v>
       </c>
       <c r="C93" t="str">
-        <v>5/5/2026, 3:24:59 pm</v>
+        <v>7/5/2026, 12:03:42 am</v>
       </c>
       <c r="D93" t="str">
-        <v>5/5/2026, 3:25:03 pm</v>
+        <v>7/5/2026, 12:03:44 am</v>
       </c>
       <c r="E93" t="str">
         <v>Success</v>
@@ -1986,16 +1986,16 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>https://www.softwebsolutions.com/automated-data-capture-solutions/</v>
+        <v>https://www.softwebsolutions.com/microsoft-consulting-services/</v>
       </c>
       <c r="B94">
-        <v>1.57</v>
+        <v>1.27</v>
       </c>
       <c r="C94" t="str">
-        <v>5/5/2026, 3:25:10 pm</v>
+        <v>7/5/2026, 12:03:50 am</v>
       </c>
       <c r="D94" t="str">
-        <v>5/5/2026, 3:25:11 pm</v>
+        <v>7/5/2026, 12:03:51 am</v>
       </c>
       <c r="E94" t="str">
         <v>Success</v>
@@ -2003,16 +2003,16 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>https://www.softwebsolutions.com/automated-quality-control-inspection-with-ai/</v>
+        <v>https://www.softwebsolutions.com/microsoft-copilot-studio-consulting/</v>
       </c>
       <c r="B95">
-        <v>4.64</v>
+        <v>1.44</v>
       </c>
       <c r="C95" t="str">
-        <v>5/5/2026, 3:25:18 pm</v>
+        <v>7/5/2026, 12:03:58 am</v>
       </c>
       <c r="D95" t="str">
-        <v>5/5/2026, 3:25:22 pm</v>
+        <v>7/5/2026, 12:03:59 am</v>
       </c>
       <c r="E95" t="str">
         <v>Success</v>
@@ -2020,16 +2020,16 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>https://www.softwebsolutions.com/autonomous-ai-agents-development/</v>
+        <v>https://www.softwebsolutions.com/microsoft-hololens-app-development-company/</v>
       </c>
       <c r="B96">
-        <v>0.97</v>
+        <v>1.31</v>
       </c>
       <c r="C96" t="str">
-        <v>5/5/2026, 3:25:28 pm</v>
+        <v>7/5/2026, 12:04:06 am</v>
       </c>
       <c r="D96" t="str">
-        <v>5/5/2026, 3:25:29 pm</v>
+        <v>7/5/2026, 12:04:07 am</v>
       </c>
       <c r="E96" t="str">
         <v>Success</v>
@@ -2037,16 +2037,16 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>https://www.softwebsolutions.com/aws-cloud-migration-services/</v>
+        <v>https://www.softwebsolutions.com/microsoft-viva-consulting/</v>
       </c>
       <c r="B97">
-        <v>4.29</v>
+        <v>1.05</v>
       </c>
       <c r="C97" t="str">
-        <v>5/5/2026, 3:25:36 pm</v>
+        <v>7/5/2026, 12:04:13 am</v>
       </c>
       <c r="D97" t="str">
-        <v>5/5/2026, 3:25:40 pm</v>
+        <v>7/5/2026, 12:04:14 am</v>
       </c>
       <c r="E97" t="str">
         <v>Success</v>
@@ -2054,16 +2054,16 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>https://www.softwebsolutions.com/aws-data-analytics-consulting/</v>
+        <v>https://www.softwebsolutions.com/mlops-consulting-services/</v>
       </c>
       <c r="B98">
-        <v>1.21</v>
+        <v>5.46</v>
       </c>
       <c r="C98" t="str">
-        <v>5/5/2026, 3:25:47 pm</v>
+        <v>7/5/2026, 12:04:20 am</v>
       </c>
       <c r="D98" t="str">
-        <v>5/5/2026, 3:25:48 pm</v>
+        <v>7/5/2026, 12:04:26 am</v>
       </c>
       <c r="E98" t="str">
         <v>Success</v>
@@ -2071,16 +2071,16 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>https://www.softwebsolutions.com/aws-sagemaker-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/mobile-app-development/</v>
       </c>
       <c r="B99">
-        <v>1.04</v>
+        <v>1.75</v>
       </c>
       <c r="C99" t="str">
-        <v>5/5/2026, 3:25:54 pm</v>
+        <v>7/5/2026, 12:04:33 am</v>
       </c>
       <c r="D99" t="str">
-        <v>5/5/2026, 3:25:55 pm</v>
+        <v>7/5/2026, 12:04:34 am</v>
       </c>
       <c r="E99" t="str">
         <v>Success</v>
@@ -2088,16 +2088,16 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>https://www.softwebsolutions.com/aws-services/</v>
+        <v>https://www.softwebsolutions.com/mulesoft-consulting-services/</v>
       </c>
       <c r="B100">
-        <v>1.34</v>
+        <v>1.67</v>
       </c>
       <c r="C100" t="str">
-        <v>5/5/2026, 3:26:02 pm</v>
+        <v>7/5/2026, 12:04:42 am</v>
       </c>
       <c r="D100" t="str">
-        <v>5/5/2026, 3:26:03 pm</v>
+        <v>7/5/2026, 12:04:43 am</v>
       </c>
       <c r="E100" t="str">
         <v>Success</v>
@@ -2105,16 +2105,16 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>https://www.softwebsolutions.com/azure-ai-services/</v>
+        <v>https://www.softwebsolutions.com/multicloud-managed-services/</v>
       </c>
       <c r="B101">
-        <v>1.9</v>
+        <v>1.55</v>
       </c>
       <c r="C101" t="str">
-        <v>5/5/2026, 3:26:09 pm</v>
+        <v>7/5/2026, 12:04:50 am</v>
       </c>
       <c r="D101" t="str">
-        <v>5/5/2026, 3:26:11 pm</v>
+        <v>7/5/2026, 12:04:51 am</v>
       </c>
       <c r="E101" t="str">
         <v>Success</v>
@@ -2122,16 +2122,16 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>https://www.softwebsolutions.com/azure-cloud-service/</v>
+        <v>https://www.softwebsolutions.com/natural-language-processing-services/</v>
       </c>
       <c r="B102">
-        <v>6.69</v>
+        <v>7.24</v>
       </c>
       <c r="C102" t="str">
-        <v>5/5/2026, 3:26:17 pm</v>
+        <v>7/5/2026, 12:04:58 am</v>
       </c>
       <c r="D102" t="str">
-        <v>5/5/2026, 3:26:23 pm</v>
+        <v>7/5/2026, 12:05:06 am</v>
       </c>
       <c r="E102" t="str">
         <v>Success</v>
@@ -2139,16 +2139,16 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>https://www.softwebsolutions.com/azure-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/net-maui-development-services/</v>
       </c>
       <c r="B103">
-        <v>4.88</v>
+        <v>4.92</v>
       </c>
       <c r="C103" t="str">
-        <v>5/5/2026, 3:26:29 pm</v>
+        <v>7/5/2026, 12:05:12 am</v>
       </c>
       <c r="D103" t="str">
-        <v>5/5/2026, 3:26:34 pm</v>
+        <v>7/5/2026, 12:05:17 am</v>
       </c>
       <c r="E103" t="str">
         <v>Success</v>
@@ -2156,16 +2156,16 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>https://www.softwebsolutions.com/azure-data-services/</v>
+        <v>https://www.softwebsolutions.com/nodejs-application-development/</v>
       </c>
       <c r="B104">
-        <v>1.2</v>
+        <v>4.97</v>
       </c>
       <c r="C104" t="str">
-        <v>5/5/2026, 3:26:40 pm</v>
+        <v>7/5/2026, 12:05:24 am</v>
       </c>
       <c r="D104" t="str">
-        <v>5/5/2026, 3:26:41 pm</v>
+        <v>7/5/2026, 12:05:29 am</v>
       </c>
       <c r="E104" t="str">
         <v>Success</v>
@@ -2173,16 +2173,16 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>https://www.softwebsolutions.com/azure-devops-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/partner-relationship-management/</v>
       </c>
       <c r="B105">
-        <v>1.3</v>
+        <v>0.82</v>
       </c>
       <c r="C105" t="str">
-        <v>5/5/2026, 3:26:48 pm</v>
+        <v>7/5/2026, 12:05:35 am</v>
       </c>
       <c r="D105" t="str">
-        <v>5/5/2026, 3:26:50 pm</v>
+        <v>7/5/2026, 12:05:36 am</v>
       </c>
       <c r="E105" t="str">
         <v>Success</v>
@@ -2190,16 +2190,16 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>https://www.softwebsolutions.com/big-data-services/</v>
+        <v>https://www.softwebsolutions.com/power-automate-consulting/</v>
       </c>
       <c r="B106">
-        <v>5.61</v>
+        <v>10.1</v>
       </c>
       <c r="C106" t="str">
-        <v>5/5/2026, 3:26:56 pm</v>
+        <v>7/5/2026, 12:05:42 am</v>
       </c>
       <c r="D106" t="str">
-        <v>5/5/2026, 3:27:02 pm</v>
+        <v>7/5/2026, 12:05:52 am</v>
       </c>
       <c r="E106" t="str">
         <v>Success</v>
@@ -2207,16 +2207,16 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>https://www.softwebsolutions.com/business-intelligence-consulting/</v>
+        <v>https://www.softwebsolutions.com/power-bi-consulting-services/</v>
       </c>
       <c r="B107">
-        <v>4.41</v>
+        <v>9.31</v>
       </c>
       <c r="C107" t="str">
-        <v>5/5/2026, 3:27:09 pm</v>
+        <v>7/5/2026, 12:05:56 am</v>
       </c>
       <c r="D107" t="str">
-        <v>5/5/2026, 3:27:13 pm</v>
+        <v>7/5/2026, 12:06:05 am</v>
       </c>
       <c r="E107" t="str">
         <v>Success</v>
@@ -2224,16 +2224,16 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>https://www.softwebsolutions.com/business-process-automation-services/</v>
+        <v>https://www.softwebsolutions.com/power-bi-oee-dashboards/</v>
       </c>
       <c r="B108">
-        <v>4.52</v>
+        <v>5.06</v>
       </c>
       <c r="C108" t="str">
-        <v>5/5/2026, 3:27:19 pm</v>
+        <v>7/5/2026, 12:06:11 am</v>
       </c>
       <c r="D108" t="str">
-        <v>5/5/2026, 3:27:24 pm</v>
+        <v>7/5/2026, 12:06:16 am</v>
       </c>
       <c r="E108" t="str">
         <v>Success</v>
@@ -2241,16 +2241,16 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>https://www.softwebsolutions.com/client-testimonial/</v>
+        <v>https://www.softwebsolutions.com/power-platform-consulting-services/</v>
       </c>
       <c r="B109">
-        <v>3.83</v>
+        <v>13.13</v>
       </c>
       <c r="C109" t="str">
-        <v>5/5/2026, 3:27:31 pm</v>
+        <v>7/5/2026, 12:06:22 am</v>
       </c>
       <c r="D109" t="str">
-        <v>5/5/2026, 3:27:35 pm</v>
+        <v>7/5/2026, 12:06:36 am</v>
       </c>
       <c r="E109" t="str">
         <v>Success</v>
@@ -2258,16 +2258,16 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>https://www.softwebsolutions.com/cloud-application-development-services/</v>
+        <v>https://www.softwebsolutions.com/powerapps-consulting-services/</v>
       </c>
       <c r="B110">
-        <v>1.64</v>
+        <v>5.18</v>
       </c>
       <c r="C110" t="str">
-        <v>5/5/2026, 3:27:43 pm</v>
+        <v>7/5/2026, 12:06:41 am</v>
       </c>
       <c r="D110" t="str">
-        <v>5/5/2026, 3:27:45 pm</v>
+        <v>7/5/2026, 12:06:46 am</v>
       </c>
       <c r="E110" t="str">
         <v>Success</v>
@@ -2275,16 +2275,16 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>https://www.softwebsolutions.com/cloud-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/predictive-analytics-services/</v>
       </c>
       <c r="B111">
-        <v>4.07</v>
+        <v>7.34</v>
       </c>
       <c r="C111" t="str">
-        <v>5/5/2026, 3:27:51 pm</v>
+        <v>7/5/2026, 12:06:54 am</v>
       </c>
       <c r="D111" t="str">
-        <v>5/5/2026, 3:27:55 pm</v>
+        <v>7/5/2026, 12:07:02 am</v>
       </c>
       <c r="E111" t="str">
         <v>Success</v>
@@ -2292,16 +2292,16 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>https://www.softwebsolutions.com/cloud-managed-services/</v>
+        <v>https://www.softwebsolutions.com/product-engineering-service/</v>
       </c>
       <c r="B112">
-        <v>1.06</v>
+        <v>5.47</v>
       </c>
       <c r="C112" t="str">
-        <v>5/5/2026, 3:28:01 pm</v>
+        <v>7/5/2026, 12:07:08 am</v>
       </c>
       <c r="D112" t="str">
-        <v>5/5/2026, 3:28:02 pm</v>
+        <v>7/5/2026, 12:07:13 am</v>
       </c>
       <c r="E112" t="str">
         <v>Success</v>
@@ -2309,16 +2309,16 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>https://www.softwebsolutions.com/cloud-migration-services/</v>
+        <v>https://www.softwebsolutions.com/product-information-management-system/</v>
       </c>
       <c r="B113">
-        <v>1.97</v>
+        <v>1.43</v>
       </c>
       <c r="C113" t="str">
-        <v>5/5/2026, 3:28:10 pm</v>
+        <v>7/5/2026, 12:07:19 am</v>
       </c>
       <c r="D113" t="str">
-        <v>5/5/2026, 3:28:12 pm</v>
+        <v>7/5/2026, 12:07:20 am</v>
       </c>
       <c r="E113" t="str">
         <v>Success</v>
@@ -2326,16 +2326,16 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>https://www.softwebsolutions.com/cloud-transformation-services/</v>
+        <v>https://www.softwebsolutions.com/</v>
       </c>
       <c r="B114">
-        <v>5.62</v>
+        <v>7.21</v>
       </c>
       <c r="C114" t="str">
-        <v>5/5/2026, 3:28:20 pm</v>
+        <v>7/5/2026, 12:00:42 am</v>
       </c>
       <c r="D114" t="str">
-        <v>5/5/2026, 3:28:26 pm</v>
+        <v>7/5/2026, 12:00:49 am</v>
       </c>
       <c r="E114" t="str">
         <v>Success</v>
@@ -2343,16 +2343,16 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>https://www.softwebsolutions.com/computer-vision/</v>
+        <v>https://www.softwebsolutions.com/about-softweb-solutions/</v>
       </c>
       <c r="B115">
-        <v>5.09</v>
+        <v>6.49</v>
       </c>
       <c r="C115" t="str">
-        <v>5/5/2026, 3:28:32 pm</v>
+        <v>7/5/2026, 12:00:57 am</v>
       </c>
       <c r="D115" t="str">
-        <v>5/5/2026, 3:28:37 pm</v>
+        <v>7/5/2026, 12:01:03 am</v>
       </c>
       <c r="E115" t="str">
         <v>Success</v>
@@ -2360,16 +2360,16 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>https://www.softwebsolutions.com/production-line-monitoring-solution/</v>
+        <v>https://www.softwebsolutions.com/adaptive-ai-development-company/</v>
       </c>
       <c r="B116">
-        <v>3.96</v>
+        <v>5.03</v>
       </c>
       <c r="C116" t="str">
-        <v>5/5/2026, 3:22:35 pm</v>
+        <v>7/5/2026, 12:01:10 am</v>
       </c>
       <c r="D116" t="str">
-        <v>5/5/2026, 3:22:39 pm</v>
+        <v>7/5/2026, 12:01:15 am</v>
       </c>
       <c r="E116" t="str">
         <v>Success</v>
@@ -2377,16 +2377,16 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>https://www.softwebsolutions.com/python-development-services/</v>
+        <v>https://www.softwebsolutions.com/agentforce-consulting-services/</v>
       </c>
       <c r="B117">
-        <v>4.7</v>
+        <v>1.82</v>
       </c>
       <c r="C117" t="str">
-        <v>5/5/2026, 3:22:43 pm</v>
+        <v>7/5/2026, 12:01:22 am</v>
       </c>
       <c r="D117" t="str">
-        <v>5/5/2026, 3:22:47 pm</v>
+        <v>7/5/2026, 12:01:24 am</v>
       </c>
       <c r="E117" t="str">
         <v>Success</v>
@@ -2394,16 +2394,16 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>https://www.softwebsolutions.com/quality-inspection-in-manufacturing/</v>
+        <v>https://www.softwebsolutions.com/agentic-ai-services/</v>
       </c>
       <c r="B118">
-        <v>4.25</v>
+        <v>5.78</v>
       </c>
       <c r="C118" t="str">
-        <v>5/5/2026, 3:22:53 pm</v>
+        <v>7/5/2026, 12:01:31 am</v>
       </c>
       <c r="D118" t="str">
-        <v>5/5/2026, 3:22:57 pm</v>
+        <v>7/5/2026, 12:01:37 am</v>
       </c>
       <c r="E118" t="str">
         <v>Success</v>
@@ -2411,16 +2411,16 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>https://www.softwebsolutions.com/rag-as-a-service/</v>
+        <v>https://www.softwebsolutions.com/ai-agent-development-company/</v>
       </c>
       <c r="B119">
-        <v>4.32</v>
+        <v>1.84</v>
       </c>
       <c r="C119" t="str">
-        <v>5/5/2026, 3:23:02 pm</v>
+        <v>7/5/2026, 12:01:43 am</v>
       </c>
       <c r="D119" t="str">
-        <v>5/5/2026, 3:23:06 pm</v>
+        <v>7/5/2026, 12:01:45 am</v>
       </c>
       <c r="E119" t="str">
         <v>Success</v>
@@ -2428,16 +2428,16 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>https://www.softwebsolutions.com/react-native-app-development-services/</v>
+        <v>https://www.softwebsolutions.com/ai-anomaly-detection/</v>
       </c>
       <c r="B120">
-        <v>1.63</v>
+        <v>0.96</v>
       </c>
       <c r="C120" t="str">
-        <v>5/5/2026, 3:23:12 pm</v>
+        <v>7/5/2026, 12:01:52 am</v>
       </c>
       <c r="D120" t="str">
-        <v>5/5/2026, 3:23:14 pm</v>
+        <v>7/5/2026, 12:01:53 am</v>
       </c>
       <c r="E120" t="str">
         <v>Success</v>
@@ -2445,16 +2445,16 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>https://www.softwebsolutions.com/reactjs-development-services/</v>
+        <v>https://www.softwebsolutions.com/ai-automation-testing-services/</v>
       </c>
       <c r="B121">
-        <v>4.63</v>
+        <v>0.84</v>
       </c>
       <c r="C121" t="str">
-        <v>5/5/2026, 3:23:19 pm</v>
+        <v>7/5/2026, 12:01:59 am</v>
       </c>
       <c r="D121" t="str">
-        <v>5/5/2026, 3:23:24 pm</v>
+        <v>7/5/2026, 12:02:00 am</v>
       </c>
       <c r="E121" t="str">
         <v>Success</v>
@@ -2462,16 +2462,16 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>https://www.softwebsolutions.com/recommendation-system-development-services/</v>
+        <v>https://www.softwebsolutions.com/ai-chatbot-development-company/</v>
       </c>
       <c r="B122">
-        <v>4.43</v>
+        <v>5.02</v>
       </c>
       <c r="C122" t="str">
-        <v>5/5/2026, 3:23:30 pm</v>
+        <v>7/5/2026, 12:02:07 am</v>
       </c>
       <c r="D122" t="str">
-        <v>5/5/2026, 3:23:34 pm</v>
+        <v>7/5/2026, 12:02:12 am</v>
       </c>
       <c r="E122" t="str">
         <v>Success</v>
@@ -2479,16 +2479,16 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-ai-consulting/</v>
+        <v>https://www.softwebsolutions.com/ai-consulting-services/</v>
       </c>
       <c r="B123">
-        <v>4.54</v>
+        <v>5.27</v>
       </c>
       <c r="C123" t="str">
-        <v>5/5/2026, 3:23:41 pm</v>
+        <v>7/5/2026, 12:02:20 am</v>
       </c>
       <c r="D123" t="str">
-        <v>5/5/2026, 3:23:45 pm</v>
+        <v>7/5/2026, 12:02:25 am</v>
       </c>
       <c r="E123" t="str">
         <v>Success</v>
@@ -2496,16 +2496,16 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-cloud-services/</v>
+        <v>https://www.softwebsolutions.com/ai-defect-detection-visual-inspection/</v>
       </c>
       <c r="B124">
-        <v>4.79</v>
+        <v>4.92</v>
       </c>
       <c r="C124" t="str">
-        <v>5/5/2026, 3:23:53 pm</v>
+        <v>7/5/2026, 12:02:31 am</v>
       </c>
       <c r="D124" t="str">
-        <v>5/5/2026, 3:23:57 pm</v>
+        <v>7/5/2026, 12:02:36 am</v>
       </c>
       <c r="E124" t="str">
         <v>Success</v>
@@ -2513,16 +2513,16 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-commerce-cloud-services/</v>
+        <v>https://www.softwebsolutions.com/ai-development-services/</v>
       </c>
       <c r="B125">
-        <v>4.89</v>
+        <v>5.05</v>
       </c>
       <c r="C125" t="str">
-        <v>5/5/2026, 3:24:03 pm</v>
+        <v>7/5/2026, 12:02:44 am</v>
       </c>
       <c r="D125" t="str">
-        <v>5/5/2026, 3:24:07 pm</v>
+        <v>7/5/2026, 12:02:49 am</v>
       </c>
       <c r="E125" t="str">
         <v>Success</v>
@@ -2530,16 +2530,16 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/ai-powered-inventory-management/</v>
       </c>
       <c r="B126">
-        <v>6.51</v>
+        <v>1.72</v>
       </c>
       <c r="C126" t="str">
-        <v>5/5/2026, 3:24:13 pm</v>
+        <v>7/5/2026, 12:02:57 am</v>
       </c>
       <c r="D126" t="str">
-        <v>5/5/2026, 3:24:20 pm</v>
+        <v>7/5/2026, 12:02:58 am</v>
       </c>
       <c r="E126" t="str">
         <v>Success</v>
@@ -2547,16 +2547,16 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-data-cloud-services/</v>
+        <v>https://www.softwebsolutions.com/ai-prompt-engineering-services/</v>
       </c>
       <c r="B127">
-        <v>4.42</v>
+        <v>7.46</v>
       </c>
       <c r="C127" t="str">
-        <v>5/5/2026, 3:24:26 pm</v>
+        <v>7/5/2026, 12:03:05 am</v>
       </c>
       <c r="D127" t="str">
-        <v>5/5/2026, 3:24:30 pm</v>
+        <v>7/5/2026, 12:03:13 am</v>
       </c>
       <c r="E127" t="str">
         <v>Success</v>
@@ -2564,16 +2564,16 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-development-services/</v>
+        <v>https://www.softwebsolutions.com/aiops-solutions/</v>
       </c>
       <c r="B128">
-        <v>5.62</v>
+        <v>1.47</v>
       </c>
       <c r="C128" t="str">
-        <v>5/5/2026, 3:24:41 pm</v>
+        <v>7/5/2026, 12:03:18 am</v>
       </c>
       <c r="D128" t="str">
-        <v>5/5/2026, 3:24:46 pm</v>
+        <v>7/5/2026, 12:03:19 am</v>
       </c>
       <c r="E128" t="str">
         <v>Success</v>
@@ -2581,16 +2581,16 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-experience-cloud-services/</v>
+        <v>https://www.softwebsolutions.com/application-managed-services/</v>
       </c>
       <c r="B129">
-        <v>0.96</v>
+        <v>9.18</v>
       </c>
       <c r="C129" t="str">
-        <v>5/5/2026, 3:24:54 pm</v>
+        <v>7/5/2026, 12:03:25 am</v>
       </c>
       <c r="D129" t="str">
-        <v>5/5/2026, 3:24:55 pm</v>
+        <v>7/5/2026, 12:03:35 am</v>
       </c>
       <c r="E129" t="str">
         <v>Success</v>
@@ -2598,16 +2598,16 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-implementation-services/</v>
+        <v>https://www.softwebsolutions.com/automated-data-capture-solutions/</v>
       </c>
       <c r="B130">
-        <v>1.59</v>
+        <v>4.82</v>
       </c>
       <c r="C130" t="str">
-        <v>5/5/2026, 3:25:04 pm</v>
+        <v>7/5/2026, 12:03:41 am</v>
       </c>
       <c r="D130" t="str">
-        <v>5/5/2026, 3:25:06 pm</v>
+        <v>7/5/2026, 12:03:46 am</v>
       </c>
       <c r="E130" t="str">
         <v>Success</v>
@@ -2615,16 +2615,16 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-integration-services/</v>
+        <v>https://www.softwebsolutions.com/automated-quality-control-inspection-with-ai/</v>
       </c>
       <c r="B131">
-        <v>6.18</v>
+        <v>5.64</v>
       </c>
       <c r="C131" t="str">
-        <v>5/5/2026, 3:25:13 pm</v>
+        <v>7/5/2026, 12:03:51 am</v>
       </c>
       <c r="D131" t="str">
-        <v>5/5/2026, 3:25:19 pm</v>
+        <v>7/5/2026, 12:03:57 am</v>
       </c>
       <c r="E131" t="str">
         <v>Success</v>
@@ -2632,16 +2632,16 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-migration-services/</v>
+        <v>https://www.softwebsolutions.com/autonomous-ai-agents-development/</v>
       </c>
       <c r="B132">
-        <v>6.85</v>
+        <v>5.93</v>
       </c>
       <c r="C132" t="str">
-        <v>5/5/2026, 3:25:27 pm</v>
+        <v>7/5/2026, 12:04:04 am</v>
       </c>
       <c r="D132" t="str">
-        <v>5/5/2026, 3:25:33 pm</v>
+        <v>7/5/2026, 12:04:10 am</v>
       </c>
       <c r="E132" t="str">
         <v>Success</v>
@@ -2649,16 +2649,16 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-revenue-cloud-advanced/</v>
+        <v>https://www.softwebsolutions.com/aws-cloud-migration-services/</v>
       </c>
       <c r="B133">
-        <v>1.68</v>
+        <v>1.23</v>
       </c>
       <c r="C133" t="str">
-        <v>5/5/2026, 3:25:39 pm</v>
+        <v>7/5/2026, 12:04:16 am</v>
       </c>
       <c r="D133" t="str">
-        <v>5/5/2026, 3:25:41 pm</v>
+        <v>7/5/2026, 12:04:18 am</v>
       </c>
       <c r="E133" t="str">
         <v>Success</v>
@@ -2666,16 +2666,16 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-revenue-cloud-services/</v>
+        <v>https://www.softwebsolutions.com/aws-data-analytics-consulting/</v>
       </c>
       <c r="B134">
-        <v>4.87</v>
+        <v>1.18</v>
       </c>
       <c r="C134" t="str">
-        <v>5/5/2026, 3:25:47 pm</v>
+        <v>7/5/2026, 12:04:24 am</v>
       </c>
       <c r="D134" t="str">
-        <v>5/5/2026, 3:25:52 pm</v>
+        <v>7/5/2026, 12:04:25 am</v>
       </c>
       <c r="E134" t="str">
         <v>Success</v>
@@ -2683,16 +2683,16 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-sales-cloud-services/</v>
+        <v>https://www.softwebsolutions.com/aws-sagemaker-consulting-services/</v>
       </c>
       <c r="B135">
-        <v>4.39</v>
+        <v>1.16</v>
       </c>
       <c r="C135" t="str">
-        <v>5/5/2026, 3:25:58 pm</v>
+        <v>7/5/2026, 12:04:32 am</v>
       </c>
       <c r="D135" t="str">
-        <v>5/5/2026, 3:26:03 pm</v>
+        <v>7/5/2026, 12:04:33 am</v>
       </c>
       <c r="E135" t="str">
         <v>Success</v>
@@ -2700,16 +2700,16 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>https://www.softwebsolutions.com/semiconductor/</v>
+        <v>https://www.softwebsolutions.com/aws-services/</v>
       </c>
       <c r="B136">
-        <v>6.93</v>
+        <v>1.62</v>
       </c>
       <c r="C136" t="str">
-        <v>5/5/2026, 3:26:09 pm</v>
+        <v>7/5/2026, 12:04:41 am</v>
       </c>
       <c r="D136" t="str">
-        <v>5/5/2026, 3:26:16 pm</v>
+        <v>7/5/2026, 12:04:42 am</v>
       </c>
       <c r="E136" t="str">
         <v>Success</v>
@@ -2717,16 +2717,16 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>https://www.softwebsolutions.com/sharepoint-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/azure-ai-services/</v>
       </c>
       <c r="B137">
-        <v>1.69</v>
+        <v>1.22</v>
       </c>
       <c r="C137" t="str">
-        <v>5/5/2026, 3:26:22 pm</v>
+        <v>7/5/2026, 12:04:49 am</v>
       </c>
       <c r="D137" t="str">
-        <v>5/5/2026, 3:26:23 pm</v>
+        <v>7/5/2026, 12:04:50 am</v>
       </c>
       <c r="E137" t="str">
         <v>Success</v>
@@ -2734,16 +2734,16 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>https://www.softwebsolutions.com/simple-reflex-ai-agents/</v>
+        <v>https://www.softwebsolutions.com/azure-cloud-service/</v>
       </c>
       <c r="B138">
-        <v>1.36</v>
+        <v>5.57</v>
       </c>
       <c r="C138" t="str">
-        <v>5/5/2026, 3:26:29 pm</v>
+        <v>7/5/2026, 12:04:57 am</v>
       </c>
       <c r="D138" t="str">
-        <v>5/5/2026, 3:26:31 pm</v>
+        <v>7/5/2026, 12:05:03 am</v>
       </c>
       <c r="E138" t="str">
         <v>Success</v>
@@ -2751,16 +2751,16 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>https://www.softwebsolutions.com/sitecore-implementation/</v>
+        <v>https://www.softwebsolutions.com/azure-consulting-services/</v>
       </c>
       <c r="B139">
-        <v>0.94</v>
+        <v>1.81</v>
       </c>
       <c r="C139" t="str">
-        <v>5/5/2026, 3:26:37 pm</v>
+        <v>7/5/2026, 12:05:10 am</v>
       </c>
       <c r="D139" t="str">
-        <v>5/5/2026, 3:26:38 pm</v>
+        <v>7/5/2026, 12:05:12 am</v>
       </c>
       <c r="E139" t="str">
         <v>Success</v>
@@ -2768,16 +2768,16 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>https://www.softwebsolutions.com/sitecore-managed-services/</v>
+        <v>https://www.softwebsolutions.com/azure-data-services/</v>
       </c>
       <c r="B140">
-        <v>1.13</v>
+        <v>1.08</v>
       </c>
       <c r="C140" t="str">
-        <v>5/5/2026, 3:26:46 pm</v>
+        <v>7/5/2026, 12:05:18 am</v>
       </c>
       <c r="D140" t="str">
-        <v>5/5/2026, 3:26:47 pm</v>
+        <v>7/5/2026, 12:05:19 am</v>
       </c>
       <c r="E140" t="str">
         <v>Success</v>
@@ -2785,16 +2785,16 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>https://www.softwebsolutions.com/snowflake-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/azure-devops-consulting-services/</v>
       </c>
       <c r="B141">
-        <v>5.03</v>
+        <v>5.29</v>
       </c>
       <c r="C141" t="str">
-        <v>5/5/2026, 3:26:53 pm</v>
+        <v>7/5/2026, 12:05:27 am</v>
       </c>
       <c r="D141" t="str">
-        <v>5/5/2026, 3:26:59 pm</v>
+        <v>7/5/2026, 12:05:33 am</v>
       </c>
       <c r="E141" t="str">
         <v>Success</v>
@@ -2802,16 +2802,16 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>https://www.softwebsolutions.com/solutions/</v>
+        <v>https://www.softwebsolutions.com/big-data-services/</v>
       </c>
       <c r="B142">
-        <v>0.88</v>
+        <v>6.13</v>
       </c>
       <c r="C142" t="str">
-        <v>5/5/2026, 3:27:04 pm</v>
+        <v>7/5/2026, 12:05:39 am</v>
       </c>
       <c r="D142" t="str">
-        <v>5/5/2026, 3:27:05 pm</v>
+        <v>7/5/2026, 12:05:45 am</v>
       </c>
       <c r="E142" t="str">
         <v>Success</v>
@@ -2819,16 +2819,16 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>https://www.softwebsolutions.com/supply-chain-automation-solution/</v>
+        <v>https://www.softwebsolutions.com/business-intelligence-consulting/</v>
       </c>
       <c r="B143">
-        <v>1.03</v>
+        <v>6.96</v>
       </c>
       <c r="C143" t="str">
-        <v>5/5/2026, 3:27:11 pm</v>
+        <v>7/5/2026, 12:05:50 am</v>
       </c>
       <c r="D143" t="str">
-        <v>5/5/2026, 3:27:12 pm</v>
+        <v>7/5/2026, 12:05:57 am</v>
       </c>
       <c r="E143" t="str">
         <v>Success</v>
@@ -2836,16 +2836,16 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>https://www.softwebsolutions.com/supply-chain-bot-development/</v>
+        <v>https://www.softwebsolutions.com/business-process-automation-services/</v>
       </c>
       <c r="B144">
-        <v>0.89</v>
+        <v>7.59</v>
       </c>
       <c r="C144" t="str">
-        <v>5/5/2026, 3:27:18 pm</v>
+        <v>7/5/2026, 12:06:02 am</v>
       </c>
       <c r="D144" t="str">
-        <v>5/5/2026, 3:27:19 pm</v>
+        <v>7/5/2026, 12:06:09 am</v>
       </c>
       <c r="E144" t="str">
         <v>Success</v>
@@ -2853,16 +2853,16 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>https://www.softwebsolutions.com/supply-chain/</v>
+        <v>https://www.softwebsolutions.com/client-testimonial/</v>
       </c>
       <c r="B145">
-        <v>1.27</v>
+        <v>4.91</v>
       </c>
       <c r="C145" t="str">
-        <v>5/5/2026, 3:27:27 pm</v>
+        <v>7/5/2026, 12:06:15 am</v>
       </c>
       <c r="D145" t="str">
-        <v>5/5/2026, 3:27:28 pm</v>
+        <v>7/5/2026, 12:06:20 am</v>
       </c>
       <c r="E145" t="str">
         <v>Success</v>
@@ -2870,16 +2870,16 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>https://www.softwebsolutions.com/surface-defect-detection/</v>
+        <v>https://www.softwebsolutions.com/cloud-application-development-services/</v>
       </c>
       <c r="B146">
-        <v>1.15</v>
+        <v>13.24</v>
       </c>
       <c r="C146" t="str">
-        <v>5/5/2026, 3:27:34 pm</v>
+        <v>7/5/2026, 12:06:26 am</v>
       </c>
       <c r="D146" t="str">
-        <v>5/5/2026, 3:27:36 pm</v>
+        <v>7/5/2026, 12:06:39 am</v>
       </c>
       <c r="E146" t="str">
         <v>Success</v>
@@ -2887,16 +2887,16 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>https://www.softwebsolutions.com/tableau-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/cloud-consulting-services/</v>
       </c>
       <c r="B147">
-        <v>4.83</v>
+        <v>5.37</v>
       </c>
       <c r="C147" t="str">
-        <v>5/5/2026, 3:27:41 pm</v>
+        <v>7/5/2026, 12:06:44 am</v>
       </c>
       <c r="D147" t="str">
-        <v>5/5/2026, 3:27:46 pm</v>
+        <v>7/5/2026, 12:06:49 am</v>
       </c>
       <c r="E147" t="str">
         <v>Success</v>
@@ -2904,16 +2904,16 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>https://www.softwebsolutions.com/vision-based-eol-detection/</v>
+        <v>https://www.softwebsolutions.com/cloud-managed-services/</v>
       </c>
       <c r="B148">
-        <v>1.11</v>
+        <v>6.05</v>
       </c>
       <c r="C148" t="str">
-        <v>5/5/2026, 3:27:52 pm</v>
+        <v>7/5/2026, 12:06:55 am</v>
       </c>
       <c r="D148" t="str">
-        <v>5/5/2026, 3:27:53 pm</v>
+        <v>7/5/2026, 12:07:01 am</v>
       </c>
       <c r="E148" t="str">
         <v>Success</v>
@@ -2921,16 +2921,16 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>https://www.softwebsolutions.com/wafer-defect-detection/</v>
+        <v>https://www.softwebsolutions.com/cloud-migration-services/</v>
       </c>
       <c r="B149">
-        <v>1.28</v>
+        <v>2.01</v>
       </c>
       <c r="C149" t="str">
-        <v>5/5/2026, 3:27:59 pm</v>
+        <v>7/5/2026, 12:07:08 am</v>
       </c>
       <c r="D149" t="str">
-        <v>5/5/2026, 3:28:00 pm</v>
+        <v>7/5/2026, 12:07:10 am</v>
       </c>
       <c r="E149" t="str">
         <v>Success</v>
@@ -2938,16 +2938,16 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>https://www.softwebsolutions.com/web-application-development/</v>
+        <v>https://www.softwebsolutions.com/cloud-transformation-services/</v>
       </c>
       <c r="B150">
-        <v>6.06</v>
+        <v>2</v>
       </c>
       <c r="C150" t="str">
-        <v>5/5/2026, 3:28:08 pm</v>
+        <v>7/5/2026, 12:07:17 am</v>
       </c>
       <c r="D150" t="str">
-        <v>5/5/2026, 3:28:14 pm</v>
+        <v>7/5/2026, 12:07:19 am</v>
       </c>
       <c r="E150" t="str">
         <v>Success</v>
@@ -2955,16 +2955,16 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>https://www.softwebsolutions.com/wordpress-development-services/</v>
+        <v>https://www.softwebsolutions.com/computer-vision/</v>
       </c>
       <c r="B151">
-        <v>1.56</v>
+        <v>1.89</v>
       </c>
       <c r="C151" t="str">
-        <v>5/5/2026, 3:28:22 pm</v>
+        <v>7/5/2026, 12:07:24 am</v>
       </c>
       <c r="D151" t="str">
-        <v>5/5/2026, 3:28:24 pm</v>
+        <v>7/5/2026, 12:07:26 am</v>
       </c>
       <c r="E151" t="str">
         <v>Success</v>

</xml_diff>

<commit_message>
fixed spell check load time execution feature
</commit_message>
<xml_diff>
--- a/excelReport/page-load-report.xlsx
+++ b/excelReport/page-load-report.xlsx
@@ -32,12 +32,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="5">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -425,13 +421,13 @@
         <v>https://www.softwebsolutions.com/custom-net-development-services/</v>
       </c>
       <c r="B2">
-        <v>8.4</v>
+        <v>6.25</v>
       </c>
       <c r="C2" t="str">
-        <v>7/5/2026, 12:00:41 am</v>
+        <v>3/7/2026, 4:48:27 pm</v>
       </c>
       <c r="D2" t="str">
-        <v>7/5/2026, 12:00:49 am</v>
+        <v>3/7/2026, 4:48:33 pm</v>
       </c>
       <c r="E2" t="str">
         <v>Success</v>
@@ -442,13 +438,13 @@
         <v>https://www.softwebsolutions.com/custom-software-development/</v>
       </c>
       <c r="B3">
-        <v>6.14</v>
+        <v>4.5</v>
       </c>
       <c r="C3" t="str">
-        <v>7/5/2026, 12:00:55 am</v>
+        <v>3/7/2026, 4:48:39 pm</v>
       </c>
       <c r="D3" t="str">
-        <v>7/5/2026, 12:01:01 am</v>
+        <v>3/7/2026, 4:48:43 pm</v>
       </c>
       <c r="E3" t="str">
         <v>Success</v>
@@ -459,13 +455,13 @@
         <v>https://www.softwebsolutions.com/customer-care-bot-development/</v>
       </c>
       <c r="B4">
-        <v>1.99</v>
+        <v>6.28</v>
       </c>
       <c r="C4" t="str">
-        <v>7/5/2026, 12:01:09 am</v>
+        <v>3/7/2026, 4:48:49 pm</v>
       </c>
       <c r="D4" t="str">
-        <v>7/5/2026, 12:01:11 am</v>
+        <v>3/7/2026, 4:48:55 pm</v>
       </c>
       <c r="E4" t="str">
         <v>Success</v>
@@ -476,13 +472,13 @@
         <v>https://www.softwebsolutions.com/customer-data-platform/</v>
       </c>
       <c r="B5">
-        <v>5.48</v>
+        <v>4.92</v>
       </c>
       <c r="C5" t="str">
-        <v>7/5/2026, 12:01:18 am</v>
+        <v>3/7/2026, 4:49:01 pm</v>
       </c>
       <c r="D5" t="str">
-        <v>7/5/2026, 12:01:23 am</v>
+        <v>3/7/2026, 4:49:06 pm</v>
       </c>
       <c r="E5" t="str">
         <v>Success</v>
@@ -493,13 +489,13 @@
         <v>https://www.softwebsolutions.com/dashboard-development-services/</v>
       </c>
       <c r="B6">
-        <v>5.25</v>
+        <v>5</v>
       </c>
       <c r="C6" t="str">
-        <v>7/5/2026, 12:01:31 am</v>
+        <v>3/7/2026, 4:49:11 pm</v>
       </c>
       <c r="D6" t="str">
-        <v>7/5/2026, 12:01:36 am</v>
+        <v>3/7/2026, 4:49:16 pm</v>
       </c>
       <c r="E6" t="str">
         <v>Success</v>
@@ -510,13 +506,13 @@
         <v>https://www.softwebsolutions.com/data-analytics-banking-dashboard/</v>
       </c>
       <c r="B7">
-        <v>4.73</v>
+        <v>1.16</v>
       </c>
       <c r="C7" t="str">
-        <v>7/5/2026, 12:01:43 am</v>
+        <v>3/7/2026, 4:49:22 pm</v>
       </c>
       <c r="D7" t="str">
-        <v>7/5/2026, 12:01:48 am</v>
+        <v>3/7/2026, 4:49:23 pm</v>
       </c>
       <c r="E7" t="str">
         <v>Success</v>
@@ -527,13 +523,13 @@
         <v>https://www.softwebsolutions.com/data-analytics-finance-dashboard/</v>
       </c>
       <c r="B8">
-        <v>1.43</v>
+        <v>6.29</v>
       </c>
       <c r="C8" t="str">
-        <v>7/5/2026, 12:01:54 am</v>
+        <v>3/7/2026, 4:49:29 pm</v>
       </c>
       <c r="D8" t="str">
-        <v>7/5/2026, 12:01:55 am</v>
+        <v>3/7/2026, 4:49:35 pm</v>
       </c>
       <c r="E8" t="str">
         <v>Success</v>
@@ -544,13 +540,13 @@
         <v>https://www.softwebsolutions.com/data-analytics-services/</v>
       </c>
       <c r="B9">
-        <v>4.39</v>
+        <v>2.2</v>
       </c>
       <c r="C9" t="str">
-        <v>7/5/2026, 12:02:01 am</v>
+        <v>3/7/2026, 4:49:41 pm</v>
       </c>
       <c r="D9" t="str">
-        <v>7/5/2026, 12:02:06 am</v>
+        <v>3/7/2026, 4:49:43 pm</v>
       </c>
       <c r="E9" t="str">
         <v>Success</v>
@@ -561,13 +557,13 @@
         <v>https://www.softwebsolutions.com/data-engineering-consulting-services/</v>
       </c>
       <c r="B10">
-        <v>4.46</v>
+        <v>5.26</v>
       </c>
       <c r="C10" t="str">
-        <v>7/5/2026, 12:02:11 am</v>
+        <v>3/7/2026, 4:49:48 pm</v>
       </c>
       <c r="D10" t="str">
-        <v>7/5/2026, 12:02:16 am</v>
+        <v>3/7/2026, 4:49:54 pm</v>
       </c>
       <c r="E10" t="str">
         <v>Success</v>
@@ -578,13 +574,13 @@
         <v>https://www.softwebsolutions.com/data-governance-services/</v>
       </c>
       <c r="B11">
-        <v>2.13</v>
+        <v>7.7</v>
       </c>
       <c r="C11" t="str">
-        <v>7/5/2026, 12:02:22 am</v>
+        <v>3/7/2026, 4:50:00 pm</v>
       </c>
       <c r="D11" t="str">
-        <v>7/5/2026, 12:02:25 am</v>
+        <v>3/7/2026, 4:50:07 pm</v>
       </c>
       <c r="E11" t="str">
         <v>Success</v>
@@ -595,13 +591,13 @@
         <v>https://www.softwebsolutions.com/data-integration-services/</v>
       </c>
       <c r="B12">
-        <v>1.42</v>
+        <v>7.82</v>
       </c>
       <c r="C12" t="str">
-        <v>7/5/2026, 12:02:31 am</v>
+        <v>3/7/2026, 4:50:13 pm</v>
       </c>
       <c r="D12" t="str">
-        <v>7/5/2026, 12:02:33 am</v>
+        <v>3/7/2026, 4:50:21 pm</v>
       </c>
       <c r="E12" t="str">
         <v>Success</v>
@@ -612,13 +608,13 @@
         <v>https://www.softwebsolutions.com/data-managed-services/</v>
       </c>
       <c r="B13">
-        <v>4.99</v>
+        <v>7.03</v>
       </c>
       <c r="C13" t="str">
-        <v>7/5/2026, 12:02:39 am</v>
+        <v>3/7/2026, 4:50:28 pm</v>
       </c>
       <c r="D13" t="str">
-        <v>7/5/2026, 12:02:44 am</v>
+        <v>3/7/2026, 4:50:35 pm</v>
       </c>
       <c r="E13" t="str">
         <v>Success</v>
@@ -629,13 +625,13 @@
         <v>https://www.softwebsolutions.com/data-migration-services/</v>
       </c>
       <c r="B14">
-        <v>4.52</v>
+        <v>7.14</v>
       </c>
       <c r="C14" t="str">
-        <v>7/5/2026, 12:02:50 am</v>
+        <v>3/7/2026, 4:51:03 pm</v>
       </c>
       <c r="D14" t="str">
-        <v>7/5/2026, 12:02:55 am</v>
+        <v>3/7/2026, 4:51:10 pm</v>
       </c>
       <c r="E14" t="str">
         <v>Success</v>
@@ -646,13 +642,13 @@
         <v>https://www.softwebsolutions.com/data-pipeline-automation-services/</v>
       </c>
       <c r="B15">
-        <v>1.58</v>
+        <v>5.73</v>
       </c>
       <c r="C15" t="str">
-        <v>7/5/2026, 12:03:01 am</v>
+        <v>3/7/2026, 4:51:18 pm</v>
       </c>
       <c r="D15" t="str">
-        <v>7/5/2026, 12:03:03 am</v>
+        <v>3/7/2026, 4:51:23 pm</v>
       </c>
       <c r="E15" t="str">
         <v>Success</v>
@@ -663,13 +659,13 @@
         <v>https://www.softwebsolutions.com/data-science-development/</v>
       </c>
       <c r="B16">
-        <v>9.58</v>
+        <v>5.93</v>
       </c>
       <c r="C16" t="str">
-        <v>7/5/2026, 12:03:08 am</v>
+        <v>3/7/2026, 4:51:30 pm</v>
       </c>
       <c r="D16" t="str">
-        <v>7/5/2026, 12:03:18 am</v>
+        <v>3/7/2026, 4:51:36 pm</v>
       </c>
       <c r="E16" t="str">
         <v>Success</v>
@@ -680,13 +676,13 @@
         <v>https://www.softwebsolutions.com/data-visualization-consulting/</v>
       </c>
       <c r="B17">
-        <v>6.92</v>
+        <v>5.64</v>
       </c>
       <c r="C17" t="str">
-        <v>7/5/2026, 12:03:24 am</v>
+        <v>3/7/2026, 4:51:41 pm</v>
       </c>
       <c r="D17" t="str">
-        <v>7/5/2026, 12:03:31 am</v>
+        <v>3/7/2026, 4:51:47 pm</v>
       </c>
       <c r="E17" t="str">
         <v>Success</v>
@@ -697,13 +693,13 @@
         <v>https://www.softwebsolutions.com/databricks-consulting-services/</v>
       </c>
       <c r="B18">
-        <v>1.04</v>
+        <v>1.77</v>
       </c>
       <c r="C18" t="str">
-        <v>7/5/2026, 12:03:36 am</v>
+        <v>3/7/2026, 4:51:52 pm</v>
       </c>
       <c r="D18" t="str">
-        <v>7/5/2026, 12:03:37 am</v>
+        <v>3/7/2026, 4:51:54 pm</v>
       </c>
       <c r="E18" t="str">
         <v>Success</v>
@@ -714,13 +710,13 @@
         <v>https://www.softwebsolutions.com/decision-intelligence-system/</v>
       </c>
       <c r="B19">
-        <v>4.84</v>
+        <v>2.35</v>
       </c>
       <c r="C19" t="str">
-        <v>7/5/2026, 12:03:43 am</v>
+        <v>3/7/2026, 4:52:00 pm</v>
       </c>
       <c r="D19" t="str">
-        <v>7/5/2026, 12:03:47 am</v>
+        <v>3/7/2026, 4:52:03 pm</v>
       </c>
       <c r="E19" t="str">
         <v>Success</v>
@@ -731,13 +727,13 @@
         <v>https://www.softwebsolutions.com/deep-learning-solutions/</v>
       </c>
       <c r="B20">
-        <v>3.89</v>
+        <v>6.02</v>
       </c>
       <c r="C20" t="str">
-        <v>7/5/2026, 12:03:53 am</v>
+        <v>3/7/2026, 4:52:09 pm</v>
       </c>
       <c r="D20" t="str">
-        <v>7/5/2026, 12:03:57 am</v>
+        <v>3/7/2026, 4:52:15 pm</v>
       </c>
       <c r="E20" t="str">
         <v>Success</v>
@@ -748,13 +744,13 @@
         <v>https://www.softwebsolutions.com/defect-detection-in-packaging/</v>
       </c>
       <c r="B21">
-        <v>5.27</v>
+        <v>4.74</v>
       </c>
       <c r="C21" t="str">
-        <v>7/5/2026, 12:04:04 am</v>
+        <v>3/7/2026, 4:52:20 pm</v>
       </c>
       <c r="D21" t="str">
-        <v>7/5/2026, 12:04:10 am</v>
+        <v>3/7/2026, 4:52:25 pm</v>
       </c>
       <c r="E21" t="str">
         <v>Success</v>
@@ -765,13 +761,13 @@
         <v>https://www.softwebsolutions.com/devops-consulting-services/</v>
       </c>
       <c r="B22">
-        <v>4.73</v>
+        <v>5.7</v>
       </c>
       <c r="C22" t="str">
-        <v>7/5/2026, 12:04:16 am</v>
+        <v>3/7/2026, 4:52:32 pm</v>
       </c>
       <c r="D22" t="str">
-        <v>7/5/2026, 12:04:21 am</v>
+        <v>3/7/2026, 4:52:37 pm</v>
       </c>
       <c r="E22" t="str">
         <v>Success</v>
@@ -782,13 +778,13 @@
         <v>https://www.softwebsolutions.com/digital-process-automation-services/</v>
       </c>
       <c r="B23">
-        <v>0.98</v>
+        <v>6.75</v>
       </c>
       <c r="C23" t="str">
-        <v>7/5/2026, 12:04:28 am</v>
+        <v>3/7/2026, 4:52:45 pm</v>
       </c>
       <c r="D23" t="str">
-        <v>7/5/2026, 12:04:29 am</v>
+        <v>3/7/2026, 4:52:51 pm</v>
       </c>
       <c r="E23" t="str">
         <v>Success</v>
@@ -799,13 +795,13 @@
         <v>https://www.softwebsolutions.com/digital-supply-chain-solutions/</v>
       </c>
       <c r="B24">
-        <v>1.13</v>
+        <v>5.7</v>
       </c>
       <c r="C24" t="str">
-        <v>7/5/2026, 12:04:35 am</v>
+        <v>3/7/2026, 4:52:57 pm</v>
       </c>
       <c r="D24" t="str">
-        <v>7/5/2026, 12:04:36 am</v>
+        <v>3/7/2026, 4:53:03 pm</v>
       </c>
       <c r="E24" t="str">
         <v>Success</v>
@@ -816,13 +812,13 @@
         <v>https://www.softwebsolutions.com/digital-supply-chain/</v>
       </c>
       <c r="B25">
-        <v>1.15</v>
+        <v>3.88</v>
       </c>
       <c r="C25" t="str">
-        <v>7/5/2026, 12:04:44 am</v>
+        <v>3/7/2026, 4:53:10 pm</v>
       </c>
       <c r="D25" t="str">
-        <v>7/5/2026, 12:04:45 am</v>
+        <v>3/7/2026, 4:53:14 pm</v>
       </c>
       <c r="E25" t="str">
         <v>Success</v>
@@ -833,13 +829,13 @@
         <v>https://www.softwebsolutions.com/digital-transformation-consulting/</v>
       </c>
       <c r="B26">
-        <v>1.53</v>
+        <v>7.11</v>
       </c>
       <c r="C26" t="str">
-        <v>7/5/2026, 12:04:51 am</v>
+        <v>3/7/2026, 4:53:23 pm</v>
       </c>
       <c r="D26" t="str">
-        <v>7/5/2026, 12:04:53 am</v>
+        <v>3/7/2026, 4:53:31 pm</v>
       </c>
       <c r="E26" t="str">
         <v>Success</v>
@@ -850,13 +846,13 @@
         <v>https://www.softwebsolutions.com/edge-ai-solutions/</v>
       </c>
       <c r="B27">
-        <v>5.3</v>
+        <v>6.47</v>
       </c>
       <c r="C27" t="str">
-        <v>7/5/2026, 12:04:59 am</v>
+        <v>3/7/2026, 4:53:38 pm</v>
       </c>
       <c r="D27" t="str">
-        <v>7/5/2026, 12:05:04 am</v>
+        <v>3/7/2026, 4:53:45 pm</v>
       </c>
       <c r="E27" t="str">
         <v>Success</v>
@@ -867,13 +863,13 @@
         <v>https://www.softwebsolutions.com/enterprise-app-development/</v>
       </c>
       <c r="B28">
-        <v>1.72</v>
+        <v>5.63</v>
       </c>
       <c r="C28" t="str">
-        <v>7/5/2026, 12:05:12 am</v>
+        <v>3/7/2026, 4:53:52 pm</v>
       </c>
       <c r="D28" t="str">
-        <v>7/5/2026, 12:05:14 am</v>
+        <v>3/7/2026, 4:53:58 pm</v>
       </c>
       <c r="E28" t="str">
         <v>Success</v>
@@ -884,13 +880,13 @@
         <v>https://www.softwebsolutions.com/enterprise-data-management-services/</v>
       </c>
       <c r="B29">
-        <v>6.1</v>
+        <v>3.42</v>
       </c>
       <c r="C29" t="str">
-        <v>7/5/2026, 12:05:19 am</v>
+        <v>3/7/2026, 4:54:06 pm</v>
       </c>
       <c r="D29" t="str">
-        <v>7/5/2026, 12:05:25 am</v>
+        <v>3/7/2026, 4:54:09 pm</v>
       </c>
       <c r="E29" t="str">
         <v>Success</v>
@@ -901,13 +897,13 @@
         <v>https://www.softwebsolutions.com/enterprise-data-warehouse/</v>
       </c>
       <c r="B30">
-        <v>4.63</v>
+        <v>6.98</v>
       </c>
       <c r="C30" t="str">
-        <v>7/5/2026, 12:05:31 am</v>
+        <v>3/7/2026, 4:54:16 pm</v>
       </c>
       <c r="D30" t="str">
-        <v>7/5/2026, 12:05:36 am</v>
+        <v>3/7/2026, 4:54:23 pm</v>
       </c>
       <c r="E30" t="str">
         <v>Success</v>
@@ -918,13 +914,13 @@
         <v>https://www.softwebsolutions.com/fabric-consulting-services/</v>
       </c>
       <c r="B31">
-        <v>8.93</v>
+        <v>7.76</v>
       </c>
       <c r="C31" t="str">
-        <v>7/5/2026, 12:05:42 am</v>
+        <v>3/7/2026, 4:54:29 pm</v>
       </c>
       <c r="D31" t="str">
-        <v>7/5/2026, 12:05:51 am</v>
+        <v>3/7/2026, 4:54:37 pm</v>
       </c>
       <c r="E31" t="str">
         <v>Success</v>
@@ -935,13 +931,13 @@
         <v>https://www.softwebsolutions.com/face-recognition-services/</v>
       </c>
       <c r="B32">
-        <v>8.92</v>
+        <v>6.54</v>
       </c>
       <c r="C32" t="str">
-        <v>7/5/2026, 12:05:56 am</v>
+        <v>3/7/2026, 4:54:45 pm</v>
       </c>
       <c r="D32" t="str">
-        <v>7/5/2026, 12:06:05 am</v>
+        <v>3/7/2026, 4:54:51 pm</v>
       </c>
       <c r="E32" t="str">
         <v>Success</v>
@@ -952,13 +948,13 @@
         <v>https://www.softwebsolutions.com/finance-industry/</v>
       </c>
       <c r="B33">
-        <v>6.37</v>
+        <v>6.77</v>
       </c>
       <c r="C33" t="str">
-        <v>7/5/2026, 12:06:11 am</v>
+        <v>3/7/2026, 4:55:07 pm</v>
       </c>
       <c r="D33" t="str">
-        <v>7/5/2026, 12:06:17 am</v>
+        <v>3/7/2026, 4:55:14 pm</v>
       </c>
       <c r="E33" t="str">
         <v>Success</v>
@@ -969,13 +965,13 @@
         <v>https://www.softwebsolutions.com/flutter-app-development-services/</v>
       </c>
       <c r="B34">
-        <v>9.8</v>
+        <v>5.24</v>
       </c>
       <c r="C34" t="str">
-        <v>7/5/2026, 12:06:22 am</v>
+        <v>3/7/2026, 4:55:21 pm</v>
       </c>
       <c r="D34" t="str">
-        <v>7/5/2026, 12:06:32 am</v>
+        <v>3/7/2026, 4:55:27 pm</v>
       </c>
       <c r="E34" t="str">
         <v>Success</v>
@@ -986,13 +982,13 @@
         <v>https://www.softwebsolutions.com/front-end-development/</v>
       </c>
       <c r="B35">
-        <v>8.39</v>
+        <v>6.05</v>
       </c>
       <c r="C35" t="str">
-        <v>7/5/2026, 12:06:35 am</v>
+        <v>3/7/2026, 4:55:31 pm</v>
       </c>
       <c r="D35" t="str">
-        <v>7/5/2026, 12:06:44 am</v>
+        <v>3/7/2026, 4:55:37 pm</v>
       </c>
       <c r="E35" t="str">
         <v>Success</v>
@@ -1003,13 +999,13 @@
         <v>https://www.softwebsolutions.com/full-stack-development-company/</v>
       </c>
       <c r="B36">
-        <v>6.66</v>
+        <v>5.64</v>
       </c>
       <c r="C36" t="str">
-        <v>7/5/2026, 12:06:52 am</v>
+        <v>3/7/2026, 4:55:42 pm</v>
       </c>
       <c r="D36" t="str">
-        <v>7/5/2026, 12:06:59 am</v>
+        <v>3/7/2026, 4:55:48 pm</v>
       </c>
       <c r="E36" t="str">
         <v>Success</v>
@@ -1020,13 +1016,13 @@
         <v>https://www.softwebsolutions.com/generative-ai-consulting-services/</v>
       </c>
       <c r="B37">
-        <v>5.87</v>
+        <v>4.01</v>
       </c>
       <c r="C37" t="str">
-        <v>7/5/2026, 12:07:06 am</v>
+        <v>3/7/2026, 4:55:52 pm</v>
       </c>
       <c r="D37" t="str">
-        <v>7/5/2026, 12:07:12 am</v>
+        <v>3/7/2026, 4:55:56 pm</v>
       </c>
       <c r="E37" t="str">
         <v>Success</v>
@@ -1037,13 +1033,13 @@
         <v>https://www.softwebsolutions.com/hybrid-cloud-services/</v>
       </c>
       <c r="B38">
-        <v>2.06</v>
+        <v>5.85</v>
       </c>
       <c r="C38" t="str">
-        <v>7/5/2026, 12:07:18 am</v>
+        <v>3/7/2026, 4:56:00 pm</v>
       </c>
       <c r="D38" t="str">
-        <v>7/5/2026, 12:07:20 am</v>
+        <v>3/7/2026, 4:56:06 pm</v>
       </c>
       <c r="E38" t="str">
         <v>Success</v>
@@ -1054,13 +1050,13 @@
         <v>https://www.softwebsolutions.com/image-annotation-services/</v>
       </c>
       <c r="B39">
-        <v>1.56</v>
+        <v>5.16</v>
       </c>
       <c r="C39" t="str">
-        <v>7/5/2026, 12:07:24 am</v>
+        <v>3/7/2026, 4:56:10 pm</v>
       </c>
       <c r="D39" t="str">
-        <v>7/5/2026, 12:07:26 am</v>
+        <v>3/7/2026, 4:56:15 pm</v>
       </c>
       <c r="E39" t="str">
         <v>Success</v>
@@ -1068,16 +1064,16 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>https://www.softwebsolutions.com/production-line-monitoring-solution/</v>
+        <v>https://www.softwebsolutions.com/</v>
       </c>
       <c r="B40">
-        <v>5.69</v>
+        <v>1.48</v>
       </c>
       <c r="C40" t="str">
-        <v>7/5/2026, 12:00:43 am</v>
+        <v>3/7/2026, 4:48:27 pm</v>
       </c>
       <c r="D40" t="str">
-        <v>7/5/2026, 12:00:49 am</v>
+        <v>3/7/2026, 4:48:28 pm</v>
       </c>
       <c r="E40" t="str">
         <v>Success</v>
@@ -1085,16 +1081,16 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>https://www.softwebsolutions.com/python-development-services/</v>
+        <v>https://www.softwebsolutions.com/about-softweb-solutions/</v>
       </c>
       <c r="B41">
-        <v>6.84</v>
+        <v>5.71</v>
       </c>
       <c r="C41" t="str">
-        <v>7/5/2026, 12:00:56 am</v>
+        <v>3/7/2026, 4:48:33 pm</v>
       </c>
       <c r="D41" t="str">
-        <v>7/5/2026, 12:01:02 am</v>
+        <v>3/7/2026, 4:48:39 pm</v>
       </c>
       <c r="E41" t="str">
         <v>Success</v>
@@ -1102,16 +1098,16 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>https://www.softwebsolutions.com/quality-inspection-in-manufacturing/</v>
+        <v>https://www.softwebsolutions.com/adaptive-ai-development-company/</v>
       </c>
       <c r="B42">
-        <v>5.2</v>
+        <v>4.51</v>
       </c>
       <c r="C42" t="str">
-        <v>7/5/2026, 12:01:10 am</v>
+        <v>3/7/2026, 4:48:48 pm</v>
       </c>
       <c r="D42" t="str">
-        <v>7/5/2026, 12:01:15 am</v>
+        <v>3/7/2026, 4:48:52 pm</v>
       </c>
       <c r="E42" t="str">
         <v>Success</v>
@@ -1119,16 +1115,16 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>https://www.softwebsolutions.com/rag-as-a-service/</v>
+        <v>https://www.softwebsolutions.com/agentforce-consulting-services/</v>
       </c>
       <c r="B43">
-        <v>1.2</v>
+        <v>3.14</v>
       </c>
       <c r="C43" t="str">
-        <v>7/5/2026, 12:01:22 am</v>
+        <v>3/7/2026, 4:48:59 pm</v>
       </c>
       <c r="D43" t="str">
-        <v>7/5/2026, 12:01:23 am</v>
+        <v>3/7/2026, 4:49:02 pm</v>
       </c>
       <c r="E43" t="str">
         <v>Success</v>
@@ -1136,16 +1132,16 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>https://www.softwebsolutions.com/react-native-app-development-services/</v>
+        <v>https://www.softwebsolutions.com/agentic-ai-services/</v>
       </c>
       <c r="B44">
-        <v>5.58</v>
+        <v>2.41</v>
       </c>
       <c r="C44" t="str">
-        <v>7/5/2026, 12:01:30 am</v>
+        <v>3/7/2026, 4:49:08 pm</v>
       </c>
       <c r="D44" t="str">
-        <v>7/5/2026, 12:01:36 am</v>
+        <v>3/7/2026, 4:49:11 pm</v>
       </c>
       <c r="E44" t="str">
         <v>Success</v>
@@ -1153,16 +1149,16 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>https://www.softwebsolutions.com/reactjs-development-services/</v>
+        <v>https://www.softwebsolutions.com/ai-agent-development-company/</v>
       </c>
       <c r="B45">
-        <v>4.84</v>
+        <v>5.28</v>
       </c>
       <c r="C45" t="str">
-        <v>7/5/2026, 12:01:42 am</v>
+        <v>3/7/2026, 4:49:15 pm</v>
       </c>
       <c r="D45" t="str">
-        <v>7/5/2026, 12:01:47 am</v>
+        <v>3/7/2026, 4:49:20 pm</v>
       </c>
       <c r="E45" t="str">
         <v>Success</v>
@@ -1170,16 +1166,16 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>https://www.softwebsolutions.com/recommendation-system-development-services/</v>
+        <v>https://www.softwebsolutions.com/ai-anomaly-detection/</v>
       </c>
       <c r="B46">
-        <v>4.84</v>
+        <v>5.37</v>
       </c>
       <c r="C46" t="str">
-        <v>7/5/2026, 12:01:53 am</v>
+        <v>3/7/2026, 4:49:26 pm</v>
       </c>
       <c r="D46" t="str">
-        <v>7/5/2026, 12:01:58 am</v>
+        <v>3/7/2026, 4:49:31 pm</v>
       </c>
       <c r="E46" t="str">
         <v>Success</v>
@@ -1187,16 +1183,16 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-ai-consulting/</v>
+        <v>https://www.softwebsolutions.com/ai-automation-testing-services/</v>
       </c>
       <c r="B47">
-        <v>5.08</v>
+        <v>5.49</v>
       </c>
       <c r="C47" t="str">
-        <v>7/5/2026, 12:02:04 am</v>
+        <v>3/7/2026, 4:49:37 pm</v>
       </c>
       <c r="D47" t="str">
-        <v>7/5/2026, 12:02:09 am</v>
+        <v>3/7/2026, 4:49:43 pm</v>
       </c>
       <c r="E47" t="str">
         <v>Success</v>
@@ -1204,16 +1200,16 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-cloud-services/</v>
+        <v>https://www.softwebsolutions.com/ai-chatbot-development-company/</v>
       </c>
       <c r="B48">
-        <v>5.11</v>
+        <v>5.64</v>
       </c>
       <c r="C48" t="str">
-        <v>7/5/2026, 12:02:16 am</v>
+        <v>3/7/2026, 4:49:48 pm</v>
       </c>
       <c r="D48" t="str">
-        <v>7/5/2026, 12:02:21 am</v>
+        <v>3/7/2026, 4:49:54 pm</v>
       </c>
       <c r="E48" t="str">
         <v>Success</v>
@@ -1221,16 +1217,16 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-commerce-cloud-services/</v>
+        <v>https://www.softwebsolutions.com/ai-consulting-services/</v>
       </c>
       <c r="B49">
-        <v>5.74</v>
+        <v>6.24</v>
       </c>
       <c r="C49" t="str">
-        <v>7/5/2026, 12:02:28 am</v>
+        <v>3/7/2026, 4:50:00 pm</v>
       </c>
       <c r="D49" t="str">
-        <v>7/5/2026, 12:02:34 am</v>
+        <v>3/7/2026, 4:50:06 pm</v>
       </c>
       <c r="E49" t="str">
         <v>Success</v>
@@ -1238,16 +1234,16 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/ai-defect-detection-visual-inspection/</v>
       </c>
       <c r="B50">
-        <v>4.78</v>
+        <v>6.5</v>
       </c>
       <c r="C50" t="str">
-        <v>7/5/2026, 12:02:42 am</v>
+        <v>3/7/2026, 4:50:13 pm</v>
       </c>
       <c r="D50" t="str">
-        <v>7/5/2026, 12:02:47 am</v>
+        <v>3/7/2026, 4:50:19 pm</v>
       </c>
       <c r="E50" t="str">
         <v>Success</v>
@@ -1255,16 +1251,16 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-data-cloud-services/</v>
+        <v>https://www.softwebsolutions.com/ai-development-services/</v>
       </c>
       <c r="B51">
-        <v>5.3</v>
+        <v>5.02</v>
       </c>
       <c r="C51" t="str">
-        <v>7/5/2026, 12:02:53 am</v>
+        <v>3/7/2026, 4:50:26 pm</v>
       </c>
       <c r="D51" t="str">
-        <v>7/5/2026, 12:02:59 am</v>
+        <v>3/7/2026, 4:50:31 pm</v>
       </c>
       <c r="E51" t="str">
         <v>Success</v>
@@ -1272,16 +1268,16 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-development-services/</v>
+        <v>https://www.softwebsolutions.com/ai-powered-inventory-management/</v>
       </c>
       <c r="B52">
-        <v>8.45</v>
+        <v>14.74</v>
       </c>
       <c r="C52" t="str">
-        <v>7/5/2026, 12:03:06 am</v>
+        <v>3/7/2026, 4:50:42 pm</v>
       </c>
       <c r="D52" t="str">
-        <v>7/5/2026, 12:03:14 am</v>
+        <v>3/7/2026, 4:50:57 pm</v>
       </c>
       <c r="E52" t="str">
         <v>Success</v>
@@ -1289,16 +1285,16 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-experience-cloud-services/</v>
+        <v>https://www.softwebsolutions.com/ai-prompt-engineering-services/</v>
       </c>
       <c r="B53">
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="C53" t="str">
-        <v>7/5/2026, 12:03:18 am</v>
+        <v>3/7/2026, 4:51:12 pm</v>
       </c>
       <c r="D53" t="str">
-        <v>7/5/2026, 12:03:20 am</v>
+        <v>3/7/2026, 4:51:20 pm</v>
       </c>
       <c r="E53" t="str">
         <v>Success</v>
@@ -1306,16 +1302,16 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-implementation-services/</v>
+        <v>https://www.softwebsolutions.com/aiops-solutions/</v>
       </c>
       <c r="B54">
-        <v>8.8</v>
+        <v>6.8</v>
       </c>
       <c r="C54" t="str">
-        <v>7/5/2026, 12:03:26 am</v>
+        <v>3/7/2026, 4:51:26 pm</v>
       </c>
       <c r="D54" t="str">
-        <v>7/5/2026, 12:03:34 am</v>
+        <v>3/7/2026, 4:51:33 pm</v>
       </c>
       <c r="E54" t="str">
         <v>Success</v>
@@ -1323,16 +1319,16 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-integration-services/</v>
+        <v>https://www.softwebsolutions.com/application-managed-services/</v>
       </c>
       <c r="B55">
-        <v>4.96</v>
+        <v>5.61</v>
       </c>
       <c r="C55" t="str">
-        <v>7/5/2026, 12:03:41 am</v>
+        <v>3/7/2026, 4:51:39 pm</v>
       </c>
       <c r="D55" t="str">
-        <v>7/5/2026, 12:03:46 am</v>
+        <v>3/7/2026, 4:51:44 pm</v>
       </c>
       <c r="E55" t="str">
         <v>Success</v>
@@ -1340,16 +1336,16 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-migration-services/</v>
+        <v>https://www.softwebsolutions.com/automated-data-capture-solutions/</v>
       </c>
       <c r="B56">
-        <v>5.57</v>
+        <v>6.41</v>
       </c>
       <c r="C56" t="str">
-        <v>7/5/2026, 12:03:52 am</v>
+        <v>3/7/2026, 4:51:49 pm</v>
       </c>
       <c r="D56" t="str">
-        <v>7/5/2026, 12:03:57 am</v>
+        <v>3/7/2026, 4:51:55 pm</v>
       </c>
       <c r="E56" t="str">
         <v>Success</v>
@@ -1357,16 +1353,16 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-revenue-cloud-advanced/</v>
+        <v>https://www.softwebsolutions.com/automated-quality-control-inspection-with-ai/</v>
       </c>
       <c r="B57">
-        <v>6.44</v>
+        <v>6.18</v>
       </c>
       <c r="C57" t="str">
-        <v>7/5/2026, 12:04:05 am</v>
+        <v>3/7/2026, 4:52:01 pm</v>
       </c>
       <c r="D57" t="str">
-        <v>7/5/2026, 12:04:11 am</v>
+        <v>3/7/2026, 4:52:07 pm</v>
       </c>
       <c r="E57" t="str">
         <v>Success</v>
@@ -1374,16 +1370,16 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-revenue-cloud-services/</v>
+        <v>https://www.softwebsolutions.com/autonomous-ai-agents-development/</v>
       </c>
       <c r="B58">
-        <v>5.19</v>
+        <v>6.32</v>
       </c>
       <c r="C58" t="str">
-        <v>7/5/2026, 12:04:18 am</v>
+        <v>3/7/2026, 4:52:12 pm</v>
       </c>
       <c r="D58" t="str">
-        <v>7/5/2026, 12:04:23 am</v>
+        <v>3/7/2026, 4:52:19 pm</v>
       </c>
       <c r="E58" t="str">
         <v>Success</v>
@@ -1391,16 +1387,16 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>https://www.softwebsolutions.com/salesforce-sales-cloud-services/</v>
+        <v>https://www.softwebsolutions.com/aws-cloud-migration-services/</v>
       </c>
       <c r="B59">
-        <v>0.95</v>
+        <v>2.4</v>
       </c>
       <c r="C59" t="str">
-        <v>7/5/2026, 12:04:29 am</v>
+        <v>3/7/2026, 4:52:24 pm</v>
       </c>
       <c r="D59" t="str">
-        <v>7/5/2026, 12:04:30 am</v>
+        <v>3/7/2026, 4:52:27 pm</v>
       </c>
       <c r="E59" t="str">
         <v>Success</v>
@@ -1408,16 +1404,16 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>https://www.softwebsolutions.com/semiconductor/</v>
+        <v>https://www.softwebsolutions.com/aws-data-analytics-consulting/</v>
       </c>
       <c r="B60">
-        <v>1.21</v>
+        <v>5.59</v>
       </c>
       <c r="C60" t="str">
-        <v>7/5/2026, 12:04:38 am</v>
+        <v>3/7/2026, 4:52:32 pm</v>
       </c>
       <c r="D60" t="str">
-        <v>7/5/2026, 12:04:39 am</v>
+        <v>3/7/2026, 4:52:38 pm</v>
       </c>
       <c r="E60" t="str">
         <v>Success</v>
@@ -1425,16 +1421,16 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>https://www.softwebsolutions.com/sharepoint-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/aws-sagemaker-consulting-services/</v>
       </c>
       <c r="B61">
-        <v>1.09</v>
+        <v>3.91</v>
       </c>
       <c r="C61" t="str">
-        <v>7/5/2026, 12:04:46 am</v>
+        <v>3/7/2026, 4:52:45 pm</v>
       </c>
       <c r="D61" t="str">
-        <v>7/5/2026, 12:04:47 am</v>
+        <v>3/7/2026, 4:52:49 pm</v>
       </c>
       <c r="E61" t="str">
         <v>Success</v>
@@ -1442,16 +1438,16 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>https://www.softwebsolutions.com/simple-reflex-ai-agents/</v>
+        <v>https://www.softwebsolutions.com/aws-services/</v>
       </c>
       <c r="B62">
-        <v>1.11</v>
+        <v>5.24</v>
       </c>
       <c r="C62" t="str">
-        <v>7/5/2026, 12:04:55 am</v>
+        <v>3/7/2026, 4:52:55 pm</v>
       </c>
       <c r="D62" t="str">
-        <v>7/5/2026, 12:04:56 am</v>
+        <v>3/7/2026, 4:53:00 pm</v>
       </c>
       <c r="E62" t="str">
         <v>Success</v>
@@ -1459,16 +1455,16 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>https://www.softwebsolutions.com/sitecore-implementation/</v>
+        <v>https://www.softwebsolutions.com/azure-ai-services/</v>
       </c>
       <c r="B63">
-        <v>1.45</v>
+        <v>5.24</v>
       </c>
       <c r="C63" t="str">
-        <v>7/5/2026, 12:05:04 am</v>
+        <v>3/7/2026, 4:53:07 pm</v>
       </c>
       <c r="D63" t="str">
-        <v>7/5/2026, 12:05:05 am</v>
+        <v>3/7/2026, 4:53:13 pm</v>
       </c>
       <c r="E63" t="str">
         <v>Success</v>
@@ -1476,16 +1472,16 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>https://www.softwebsolutions.com/sitecore-managed-services/</v>
+        <v>https://www.softwebsolutions.com/azure-cloud-service/</v>
       </c>
       <c r="B64">
-        <v>1.81</v>
+        <v>7.63</v>
       </c>
       <c r="C64" t="str">
-        <v>7/5/2026, 12:05:11 am</v>
+        <v>3/7/2026, 4:53:23 pm</v>
       </c>
       <c r="D64" t="str">
-        <v>7/5/2026, 12:05:13 am</v>
+        <v>3/7/2026, 4:53:30 pm</v>
       </c>
       <c r="E64" t="str">
         <v>Success</v>
@@ -1493,16 +1489,16 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>https://www.softwebsolutions.com/snowflake-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/azure-consulting-services/</v>
       </c>
       <c r="B65">
-        <v>5.92</v>
+        <v>4.76</v>
       </c>
       <c r="C65" t="str">
-        <v>7/5/2026, 12:05:19 am</v>
+        <v>3/7/2026, 4:53:38 pm</v>
       </c>
       <c r="D65" t="str">
-        <v>7/5/2026, 12:05:25 am</v>
+        <v>3/7/2026, 4:53:43 pm</v>
       </c>
       <c r="E65" t="str">
         <v>Success</v>
@@ -1510,16 +1506,16 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>https://www.softwebsolutions.com/solutions/</v>
+        <v>https://www.softwebsolutions.com/azure-data-services/</v>
       </c>
       <c r="B66">
-        <v>1.07</v>
+        <v>4.13</v>
       </c>
       <c r="C66" t="str">
-        <v>7/5/2026, 12:05:31 am</v>
+        <v>3/7/2026, 4:53:52 pm</v>
       </c>
       <c r="D66" t="str">
-        <v>7/5/2026, 12:05:32 am</v>
+        <v>3/7/2026, 4:53:56 pm</v>
       </c>
       <c r="E66" t="str">
         <v>Success</v>
@@ -1527,16 +1523,16 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>https://www.softwebsolutions.com/supply-chain-automation-solution/</v>
+        <v>https://www.softwebsolutions.com/azure-devops-consulting-services/</v>
       </c>
       <c r="B67">
-        <v>0.95</v>
+        <v>6.67</v>
       </c>
       <c r="C67" t="str">
-        <v>7/5/2026, 12:05:38 am</v>
+        <v>3/7/2026, 4:54:03 pm</v>
       </c>
       <c r="D67" t="str">
-        <v>7/5/2026, 12:05:39 am</v>
+        <v>3/7/2026, 4:54:10 pm</v>
       </c>
       <c r="E67" t="str">
         <v>Success</v>
@@ -1544,16 +1540,16 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>https://www.softwebsolutions.com/supply-chain-bot-development/</v>
+        <v>https://www.softwebsolutions.com/big-data-services/</v>
       </c>
       <c r="B68">
-        <v>1.61</v>
+        <v>5.37</v>
       </c>
       <c r="C68" t="str">
-        <v>7/5/2026, 12:05:45 am</v>
+        <v>3/7/2026, 4:54:16 pm</v>
       </c>
       <c r="D68" t="str">
-        <v>7/5/2026, 12:05:47 am</v>
+        <v>3/7/2026, 4:54:21 pm</v>
       </c>
       <c r="E68" t="str">
         <v>Success</v>
@@ -1561,16 +1557,16 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>https://www.softwebsolutions.com/supply-chain/</v>
+        <v>https://www.softwebsolutions.com/business-intelligence-consulting/</v>
       </c>
       <c r="B69">
-        <v>7.21</v>
+        <v>6.22</v>
       </c>
       <c r="C69" t="str">
-        <v>7/5/2026, 12:05:50 am</v>
+        <v>3/7/2026, 4:54:28 pm</v>
       </c>
       <c r="D69" t="str">
-        <v>7/5/2026, 12:05:57 am</v>
+        <v>3/7/2026, 4:54:34 pm</v>
       </c>
       <c r="E69" t="str">
         <v>Success</v>
@@ -1578,16 +1574,16 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>https://www.softwebsolutions.com/surface-defect-detection/</v>
+        <v>https://www.softwebsolutions.com/business-process-automation-services/</v>
       </c>
       <c r="B70">
-        <v>6.67</v>
+        <v>7.04</v>
       </c>
       <c r="C70" t="str">
-        <v>7/5/2026, 12:06:02 am</v>
+        <v>3/7/2026, 4:54:42 pm</v>
       </c>
       <c r="D70" t="str">
-        <v>7/5/2026, 12:06:09 am</v>
+        <v>3/7/2026, 4:54:49 pm</v>
       </c>
       <c r="E70" t="str">
         <v>Success</v>
@@ -1595,16 +1591,16 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>https://www.softwebsolutions.com/tableau-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/client-testimonial/</v>
       </c>
       <c r="B71">
-        <v>4.72</v>
+        <v>6.79</v>
       </c>
       <c r="C71" t="str">
-        <v>7/5/2026, 12:06:15 am</v>
+        <v>3/7/2026, 4:54:57 pm</v>
       </c>
       <c r="D71" t="str">
-        <v>7/5/2026, 12:06:19 am</v>
+        <v>3/7/2026, 4:55:04 pm</v>
       </c>
       <c r="E71" t="str">
         <v>Success</v>
@@ -1612,16 +1608,16 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>https://www.softwebsolutions.com/vision-based-eol-detection/</v>
+        <v>https://www.softwebsolutions.com/cloud-application-development-services/</v>
       </c>
       <c r="B72">
-        <v>14.25</v>
+        <v>21.39</v>
       </c>
       <c r="C72" t="str">
-        <v>7/5/2026, 12:06:24 am</v>
+        <v>3/7/2026, 4:55:12 pm</v>
       </c>
       <c r="D72" t="str">
-        <v>7/5/2026, 12:06:38 am</v>
+        <v>3/7/2026, 4:55:33 pm</v>
       </c>
       <c r="E72" t="str">
         <v>Success</v>
@@ -1629,16 +1625,16 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>https://www.softwebsolutions.com/wafer-defect-detection/</v>
+        <v>https://www.softwebsolutions.com/cloud-consulting-services/</v>
       </c>
       <c r="B73">
-        <v>4.91</v>
+        <v>5.52</v>
       </c>
       <c r="C73" t="str">
-        <v>7/5/2026, 12:06:43 am</v>
+        <v>3/7/2026, 4:55:38 pm</v>
       </c>
       <c r="D73" t="str">
-        <v>7/5/2026, 12:06:48 am</v>
+        <v>3/7/2026, 4:55:44 pm</v>
       </c>
       <c r="E73" t="str">
         <v>Success</v>
@@ -1646,16 +1642,16 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>https://www.softwebsolutions.com/web-application-development/</v>
+        <v>https://www.softwebsolutions.com/cloud-managed-services/</v>
       </c>
       <c r="B74">
-        <v>2.29</v>
+        <v>5.13</v>
       </c>
       <c r="C74" t="str">
-        <v>7/5/2026, 12:06:55 am</v>
+        <v>3/7/2026, 4:55:50 pm</v>
       </c>
       <c r="D74" t="str">
-        <v>7/5/2026, 12:06:57 am</v>
+        <v>3/7/2026, 4:55:55 pm</v>
       </c>
       <c r="E74" t="str">
         <v>Success</v>
@@ -1663,16 +1659,16 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>https://www.softwebsolutions.com/wordpress-development-services/</v>
+        <v>https://www.softwebsolutions.com/cloud-migration-services/</v>
       </c>
       <c r="B75">
-        <v>2.17</v>
+        <v>5.05</v>
       </c>
       <c r="C75" t="str">
-        <v>7/5/2026, 12:07:06 am</v>
+        <v>3/7/2026, 4:56:00 pm</v>
       </c>
       <c r="D75" t="str">
-        <v>7/5/2026, 12:07:08 am</v>
+        <v>3/7/2026, 4:56:05 pm</v>
       </c>
       <c r="E75" t="str">
         <v>Success</v>
@@ -1680,16 +1676,16 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>https://www.softwebsolutions.com/image-processing-services/</v>
+        <v>https://www.softwebsolutions.com/cloud-transformation-services/</v>
       </c>
       <c r="B76">
-        <v>6.01</v>
+        <v>2.56</v>
       </c>
       <c r="C76" t="str">
-        <v>7/5/2026, 12:00:43 am</v>
+        <v>3/7/2026, 4:56:09 pm</v>
       </c>
       <c r="D76" t="str">
-        <v>7/5/2026, 12:00:49 am</v>
+        <v>3/7/2026, 4:56:11 pm</v>
       </c>
       <c r="E76" t="str">
         <v>Success</v>
@@ -1697,16 +1693,16 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>https://www.softwebsolutions.com/industries/</v>
+        <v>https://www.softwebsolutions.com/computer-vision/</v>
       </c>
       <c r="B77">
-        <v>6.02</v>
+        <v>4.85</v>
       </c>
       <c r="C77" t="str">
-        <v>7/5/2026, 12:00:56 am</v>
+        <v>3/7/2026, 4:56:15 pm</v>
       </c>
       <c r="D77" t="str">
-        <v>7/5/2026, 12:01:02 am</v>
+        <v>3/7/2026, 4:56:20 pm</v>
       </c>
       <c r="E77" t="str">
         <v>Success</v>
@@ -1714,16 +1710,16 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>https://www.softwebsolutions.com/intelligent-automation-services/</v>
+        <v>https://www.softwebsolutions.com/image-processing-services/</v>
       </c>
       <c r="B78">
-        <v>1.57</v>
+        <v>4.68</v>
       </c>
       <c r="C78" t="str">
-        <v>7/5/2026, 12:01:09 am</v>
+        <v>3/7/2026, 4:48:28 pm</v>
       </c>
       <c r="D78" t="str">
-        <v>7/5/2026, 12:01:11 am</v>
+        <v>3/7/2026, 4:48:33 pm</v>
       </c>
       <c r="E78" t="str">
         <v>Success</v>
@@ -1731,16 +1727,16 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>https://www.softwebsolutions.com/intelligent-document-processing-solutions/</v>
+        <v>https://www.softwebsolutions.com/industries/</v>
       </c>
       <c r="B79">
-        <v>1.46</v>
+        <v>5.71</v>
       </c>
       <c r="C79" t="str">
-        <v>7/5/2026, 12:01:19 am</v>
+        <v>3/7/2026, 4:48:38 pm</v>
       </c>
       <c r="D79" t="str">
-        <v>7/5/2026, 12:01:21 am</v>
+        <v>3/7/2026, 4:48:44 pm</v>
       </c>
       <c r="E79" t="str">
         <v>Success</v>
@@ -1748,16 +1744,16 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>https://www.softwebsolutions.com/intelligent-forecasting-services/</v>
+        <v>https://www.softwebsolutions.com/intelligent-automation-services/</v>
       </c>
       <c r="B80">
-        <v>4.99</v>
+        <v>6.22</v>
       </c>
       <c r="C80" t="str">
-        <v>7/5/2026, 12:01:28 am</v>
+        <v>3/7/2026, 4:48:49 pm</v>
       </c>
       <c r="D80" t="str">
-        <v>7/5/2026, 12:01:33 am</v>
+        <v>3/7/2026, 4:48:56 pm</v>
       </c>
       <c r="E80" t="str">
         <v>Success</v>
@@ -1765,16 +1761,16 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>https://www.softwebsolutions.com/intelligent-video-analytics-solutions/</v>
+        <v>https://www.softwebsolutions.com/intelligent-document-processing-solutions/</v>
       </c>
       <c r="B81">
-        <v>0.99</v>
+        <v>20.05</v>
       </c>
       <c r="C81" t="str">
-        <v>7/5/2026, 12:01:40 am</v>
+        <v>3/7/2026, 4:49:02 pm</v>
       </c>
       <c r="D81" t="str">
-        <v>7/5/2026, 12:01:41 am</v>
+        <v>3/7/2026, 4:49:22 pm</v>
       </c>
       <c r="E81" t="str">
         <v>Success</v>
@@ -1782,16 +1778,16 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>https://www.softwebsolutions.com/intelligent-virtual-assistant/</v>
+        <v>https://www.softwebsolutions.com/intelligent-forecasting-services/</v>
       </c>
       <c r="B82">
-        <v>4.91</v>
+        <v>4.54</v>
       </c>
       <c r="C82" t="str">
-        <v>7/5/2026, 12:01:50 am</v>
+        <v>3/7/2026, 4:49:27 pm</v>
       </c>
       <c r="D82" t="str">
-        <v>7/5/2026, 12:01:55 am</v>
+        <v>3/7/2026, 4:49:32 pm</v>
       </c>
       <c r="E82" t="str">
         <v>Success</v>
@@ -1799,16 +1795,16 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>https://www.softwebsolutions.com/inventory-analytics-dashboards/</v>
+        <v>https://www.softwebsolutions.com/intelligent-video-analytics-solutions/</v>
       </c>
       <c r="B83">
-        <v>1.5</v>
+        <v>6.37</v>
       </c>
       <c r="C83" t="str">
-        <v>7/5/2026, 12:02:02 am</v>
+        <v>3/7/2026, 4:49:37 pm</v>
       </c>
       <c r="D83" t="str">
-        <v>7/5/2026, 12:02:04 am</v>
+        <v>3/7/2026, 4:49:43 pm</v>
       </c>
       <c r="E83" t="str">
         <v>Success</v>
@@ -1816,16 +1812,16 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>https://www.softwebsolutions.com/large-language-model-development/</v>
+        <v>https://www.softwebsolutions.com/intelligent-virtual-assistant/</v>
       </c>
       <c r="B84">
-        <v>5.97</v>
+        <v>6.53</v>
       </c>
       <c r="C84" t="str">
-        <v>7/5/2026, 12:02:09 am</v>
+        <v>3/7/2026, 4:49:49 pm</v>
       </c>
       <c r="D84" t="str">
-        <v>7/5/2026, 12:02:15 am</v>
+        <v>3/7/2026, 4:49:55 pm</v>
       </c>
       <c r="E84" t="str">
         <v>Success</v>
@@ -1833,16 +1829,16 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>https://www.softwebsolutions.com/legacy-application-modernization/</v>
+        <v>https://www.softwebsolutions.com/inventory-analytics-dashboards/</v>
       </c>
       <c r="B85">
-        <v>1.21</v>
+        <v>6.36</v>
       </c>
       <c r="C85" t="str">
-        <v>7/5/2026, 12:02:22 am</v>
+        <v>3/7/2026, 4:50:00 pm</v>
       </c>
       <c r="D85" t="str">
-        <v>7/5/2026, 12:02:24 am</v>
+        <v>3/7/2026, 4:50:07 pm</v>
       </c>
       <c r="E85" t="str">
         <v>Success</v>
@@ -1850,16 +1846,16 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>https://www.softwebsolutions.com/llmops-services/</v>
+        <v>https://www.softwebsolutions.com/large-language-model-development/</v>
       </c>
       <c r="B86">
-        <v>1.2</v>
+        <v>7.65</v>
       </c>
       <c r="C86" t="str">
-        <v>7/5/2026, 12:02:30 am</v>
+        <v>3/7/2026, 4:50:13 pm</v>
       </c>
       <c r="D86" t="str">
-        <v>7/5/2026, 12:02:31 am</v>
+        <v>3/7/2026, 4:50:20 pm</v>
       </c>
       <c r="E86" t="str">
         <v>Success</v>
@@ -1867,16 +1863,16 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>https://www.softwebsolutions.com/machine-learning-consulting/</v>
+        <v>https://www.softwebsolutions.com/legacy-application-modernization/</v>
       </c>
       <c r="B87">
-        <v>1.53</v>
+        <v>6.89</v>
       </c>
       <c r="C87" t="str">
-        <v>7/5/2026, 12:02:39 am</v>
+        <v>3/7/2026, 4:50:27 pm</v>
       </c>
       <c r="D87" t="str">
-        <v>7/5/2026, 12:02:40 am</v>
+        <v>3/7/2026, 4:50:34 pm</v>
       </c>
       <c r="E87" t="str">
         <v>Success</v>
@@ -1884,16 +1880,16 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>https://www.softwebsolutions.com/machine-learning-services/</v>
+        <v>https://www.softwebsolutions.com/llmops-services/</v>
       </c>
       <c r="B88">
-        <v>1.34</v>
+        <v>12.37</v>
       </c>
       <c r="C88" t="str">
-        <v>7/5/2026, 12:02:48 am</v>
+        <v>3/7/2026, 4:50:46 pm</v>
       </c>
       <c r="D88" t="str">
-        <v>7/5/2026, 12:02:49 am</v>
+        <v>3/7/2026, 4:50:58 pm</v>
       </c>
       <c r="E88" t="str">
         <v>Success</v>
@@ -1901,16 +1897,16 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>https://www.softwebsolutions.com/machine-monitoring-system/</v>
+        <v>https://www.softwebsolutions.com/machine-learning-consulting/</v>
       </c>
       <c r="B89">
-        <v>5.09</v>
+        <v>6.56</v>
       </c>
       <c r="C89" t="str">
-        <v>7/5/2026, 12:02:57 am</v>
+        <v>3/7/2026, 4:51:14 pm</v>
       </c>
       <c r="D89" t="str">
-        <v>7/5/2026, 12:03:02 am</v>
+        <v>3/7/2026, 4:51:21 pm</v>
       </c>
       <c r="E89" t="str">
         <v>Success</v>
@@ -1918,16 +1914,16 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>https://www.softwebsolutions.com/managed-services-provider/</v>
+        <v>https://www.softwebsolutions.com/machine-learning-services/</v>
       </c>
       <c r="B90">
-        <v>5.97</v>
+        <v>6.14</v>
       </c>
       <c r="C90" t="str">
-        <v>7/5/2026, 12:03:09 am</v>
+        <v>3/7/2026, 4:51:26 pm</v>
       </c>
       <c r="D90" t="str">
-        <v>7/5/2026, 12:03:15 am</v>
+        <v>3/7/2026, 4:51:33 pm</v>
       </c>
       <c r="E90" t="str">
         <v>Success</v>
@@ -1935,16 +1931,16 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>https://www.softwebsolutions.com/manufacturing-industry/</v>
+        <v>https://www.softwebsolutions.com/machine-monitoring-system/</v>
       </c>
       <c r="B91">
-        <v>1.59</v>
+        <v>7.02</v>
       </c>
       <c r="C91" t="str">
-        <v>7/5/2026, 12:03:20 am</v>
+        <v>3/7/2026, 4:51:39 pm</v>
       </c>
       <c r="D91" t="str">
-        <v>7/5/2026, 12:03:21 am</v>
+        <v>3/7/2026, 4:51:46 pm</v>
       </c>
       <c r="E91" t="str">
         <v>Success</v>
@@ -1952,16 +1948,16 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>https://www.softwebsolutions.com/microservices/</v>
+        <v>https://www.softwebsolutions.com/managed-services-provider/</v>
       </c>
       <c r="B92">
-        <v>9.09</v>
+        <v>5.73</v>
       </c>
       <c r="C92" t="str">
-        <v>7/5/2026, 12:03:27 am</v>
+        <v>3/7/2026, 4:51:52 pm</v>
       </c>
       <c r="D92" t="str">
-        <v>7/5/2026, 12:03:36 am</v>
+        <v>3/7/2026, 4:51:58 pm</v>
       </c>
       <c r="E92" t="str">
         <v>Success</v>
@@ -1969,16 +1965,16 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>https://www.softwebsolutions.com/microsoft-365-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/manufacturing-industry/</v>
       </c>
       <c r="B93">
-        <v>1.69</v>
+        <v>4.68</v>
       </c>
       <c r="C93" t="str">
-        <v>7/5/2026, 12:03:42 am</v>
+        <v>3/7/2026, 4:52:04 pm</v>
       </c>
       <c r="D93" t="str">
-        <v>7/5/2026, 12:03:44 am</v>
+        <v>3/7/2026, 4:52:09 pm</v>
       </c>
       <c r="E93" t="str">
         <v>Success</v>
@@ -1986,16 +1982,16 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>https://www.softwebsolutions.com/microsoft-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/microservices/</v>
       </c>
       <c r="B94">
-        <v>1.27</v>
+        <v>6.14</v>
       </c>
       <c r="C94" t="str">
-        <v>7/5/2026, 12:03:50 am</v>
+        <v>3/7/2026, 4:52:14 pm</v>
       </c>
       <c r="D94" t="str">
-        <v>7/5/2026, 12:03:51 am</v>
+        <v>3/7/2026, 4:52:20 pm</v>
       </c>
       <c r="E94" t="str">
         <v>Success</v>
@@ -2003,16 +1999,16 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>https://www.softwebsolutions.com/microsoft-copilot-studio-consulting/</v>
+        <v>https://www.softwebsolutions.com/microsoft-365-consulting-services/</v>
       </c>
       <c r="B95">
-        <v>1.44</v>
+        <v>6</v>
       </c>
       <c r="C95" t="str">
-        <v>7/5/2026, 12:03:58 am</v>
+        <v>3/7/2026, 4:52:25 pm</v>
       </c>
       <c r="D95" t="str">
-        <v>7/5/2026, 12:03:59 am</v>
+        <v>3/7/2026, 4:52:31 pm</v>
       </c>
       <c r="E95" t="str">
         <v>Success</v>
@@ -2020,16 +2016,16 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>https://www.softwebsolutions.com/microsoft-hololens-app-development-company/</v>
+        <v>https://www.softwebsolutions.com/microsoft-consulting-services/</v>
       </c>
       <c r="B96">
-        <v>1.31</v>
+        <v>5.4</v>
       </c>
       <c r="C96" t="str">
-        <v>7/5/2026, 12:04:06 am</v>
+        <v>3/7/2026, 4:52:37 pm</v>
       </c>
       <c r="D96" t="str">
-        <v>7/5/2026, 12:04:07 am</v>
+        <v>3/7/2026, 4:52:43 pm</v>
       </c>
       <c r="E96" t="str">
         <v>Success</v>
@@ -2037,16 +2033,16 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>https://www.softwebsolutions.com/microsoft-viva-consulting/</v>
+        <v>https://www.softwebsolutions.com/microsoft-copilot-studio-consulting/</v>
       </c>
       <c r="B97">
-        <v>1.05</v>
+        <v>5.42</v>
       </c>
       <c r="C97" t="str">
-        <v>7/5/2026, 12:04:13 am</v>
+        <v>3/7/2026, 4:52:50 pm</v>
       </c>
       <c r="D97" t="str">
-        <v>7/5/2026, 12:04:14 am</v>
+        <v>3/7/2026, 4:52:55 pm</v>
       </c>
       <c r="E97" t="str">
         <v>Success</v>
@@ -2054,16 +2050,16 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>https://www.softwebsolutions.com/mlops-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/microsoft-hololens-app-development-company/</v>
       </c>
       <c r="B98">
-        <v>5.46</v>
+        <v>5.83</v>
       </c>
       <c r="C98" t="str">
-        <v>7/5/2026, 12:04:20 am</v>
+        <v>3/7/2026, 4:53:02 pm</v>
       </c>
       <c r="D98" t="str">
-        <v>7/5/2026, 12:04:26 am</v>
+        <v>3/7/2026, 4:53:08 pm</v>
       </c>
       <c r="E98" t="str">
         <v>Success</v>
@@ -2071,16 +2067,16 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>https://www.softwebsolutions.com/mobile-app-development/</v>
+        <v>https://www.softwebsolutions.com/microsoft-viva-consulting/</v>
       </c>
       <c r="B99">
-        <v>1.75</v>
+        <v>5.15</v>
       </c>
       <c r="C99" t="str">
-        <v>7/5/2026, 12:04:33 am</v>
+        <v>3/7/2026, 4:53:17 pm</v>
       </c>
       <c r="D99" t="str">
-        <v>7/5/2026, 12:04:34 am</v>
+        <v>3/7/2026, 4:53:22 pm</v>
       </c>
       <c r="E99" t="str">
         <v>Success</v>
@@ -2088,16 +2084,16 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>https://www.softwebsolutions.com/mulesoft-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/mlops-consulting-services/</v>
       </c>
       <c r="B100">
-        <v>1.67</v>
+        <v>8.78</v>
       </c>
       <c r="C100" t="str">
-        <v>7/5/2026, 12:04:42 am</v>
+        <v>3/7/2026, 4:53:35 pm</v>
       </c>
       <c r="D100" t="str">
-        <v>7/5/2026, 12:04:43 am</v>
+        <v>3/7/2026, 4:53:44 pm</v>
       </c>
       <c r="E100" t="str">
         <v>Success</v>
@@ -2105,16 +2101,16 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>https://www.softwebsolutions.com/multicloud-managed-services/</v>
+        <v>https://www.softwebsolutions.com/mobile-app-development/</v>
       </c>
       <c r="B101">
-        <v>1.55</v>
+        <v>7.39</v>
       </c>
       <c r="C101" t="str">
-        <v>7/5/2026, 12:04:50 am</v>
+        <v>3/7/2026, 4:53:52 pm</v>
       </c>
       <c r="D101" t="str">
-        <v>7/5/2026, 12:04:51 am</v>
+        <v>3/7/2026, 4:53:59 pm</v>
       </c>
       <c r="E101" t="str">
         <v>Success</v>
@@ -2122,16 +2118,16 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>https://www.softwebsolutions.com/natural-language-processing-services/</v>
+        <v>https://www.softwebsolutions.com/mulesoft-consulting-services/</v>
       </c>
       <c r="B102">
-        <v>7.24</v>
+        <v>5.46</v>
       </c>
       <c r="C102" t="str">
-        <v>7/5/2026, 12:04:58 am</v>
+        <v>3/7/2026, 4:54:07 pm</v>
       </c>
       <c r="D102" t="str">
-        <v>7/5/2026, 12:05:06 am</v>
+        <v>3/7/2026, 4:54:13 pm</v>
       </c>
       <c r="E102" t="str">
         <v>Success</v>
@@ -2139,16 +2135,16 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>https://www.softwebsolutions.com/net-maui-development-services/</v>
+        <v>https://www.softwebsolutions.com/multicloud-managed-services/</v>
       </c>
       <c r="B103">
-        <v>4.92</v>
+        <v>2.65</v>
       </c>
       <c r="C103" t="str">
-        <v>7/5/2026, 12:05:12 am</v>
+        <v>3/7/2026, 4:54:20 pm</v>
       </c>
       <c r="D103" t="str">
-        <v>7/5/2026, 12:05:17 am</v>
+        <v>3/7/2026, 4:54:22 pm</v>
       </c>
       <c r="E103" t="str">
         <v>Success</v>
@@ -2156,16 +2152,16 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>https://www.softwebsolutions.com/nodejs-application-development/</v>
+        <v>https://www.softwebsolutions.com/natural-language-processing-services/</v>
       </c>
       <c r="B104">
-        <v>4.97</v>
+        <v>8.13</v>
       </c>
       <c r="C104" t="str">
-        <v>7/5/2026, 12:05:24 am</v>
+        <v>3/7/2026, 4:54:29 pm</v>
       </c>
       <c r="D104" t="str">
-        <v>7/5/2026, 12:05:29 am</v>
+        <v>3/7/2026, 4:54:37 pm</v>
       </c>
       <c r="E104" t="str">
         <v>Success</v>
@@ -2173,16 +2169,16 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>https://www.softwebsolutions.com/partner-relationship-management/</v>
+        <v>https://www.softwebsolutions.com/net-maui-development-services/</v>
       </c>
       <c r="B105">
-        <v>0.82</v>
+        <v>2.08</v>
       </c>
       <c r="C105" t="str">
-        <v>7/5/2026, 12:05:35 am</v>
+        <v>3/7/2026, 4:54:45 pm</v>
       </c>
       <c r="D105" t="str">
-        <v>7/5/2026, 12:05:36 am</v>
+        <v>3/7/2026, 4:54:47 pm</v>
       </c>
       <c r="E105" t="str">
         <v>Success</v>
@@ -2190,16 +2186,16 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>https://www.softwebsolutions.com/power-automate-consulting/</v>
+        <v>https://www.softwebsolutions.com/nodejs-application-development/</v>
       </c>
       <c r="B106">
-        <v>10.1</v>
+        <v>6.54</v>
       </c>
       <c r="C106" t="str">
-        <v>7/5/2026, 12:05:42 am</v>
+        <v>3/7/2026, 4:54:56 pm</v>
       </c>
       <c r="D106" t="str">
-        <v>7/5/2026, 12:05:52 am</v>
+        <v>3/7/2026, 4:55:03 pm</v>
       </c>
       <c r="E106" t="str">
         <v>Success</v>
@@ -2207,16 +2203,16 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>https://www.softwebsolutions.com/power-bi-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/partner-relationship-management/</v>
       </c>
       <c r="B107">
-        <v>9.31</v>
+        <v>6.97</v>
       </c>
       <c r="C107" t="str">
-        <v>7/5/2026, 12:05:56 am</v>
+        <v>3/7/2026, 4:55:11 pm</v>
       </c>
       <c r="D107" t="str">
-        <v>7/5/2026, 12:06:05 am</v>
+        <v>3/7/2026, 4:55:18 pm</v>
       </c>
       <c r="E107" t="str">
         <v>Success</v>
@@ -2224,16 +2220,16 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>https://www.softwebsolutions.com/power-bi-oee-dashboards/</v>
+        <v>https://www.softwebsolutions.com/power-automate-consulting/</v>
       </c>
       <c r="B108">
-        <v>5.06</v>
+        <v>2.96</v>
       </c>
       <c r="C108" t="str">
-        <v>7/5/2026, 12:06:11 am</v>
+        <v>3/7/2026, 4:55:23 pm</v>
       </c>
       <c r="D108" t="str">
-        <v>7/5/2026, 12:06:16 am</v>
+        <v>3/7/2026, 4:55:26 pm</v>
       </c>
       <c r="E108" t="str">
         <v>Success</v>
@@ -2241,16 +2237,16 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>https://www.softwebsolutions.com/power-platform-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/power-bi-consulting-services/</v>
       </c>
       <c r="B109">
-        <v>13.13</v>
+        <v>5.12</v>
       </c>
       <c r="C109" t="str">
-        <v>7/5/2026, 12:06:22 am</v>
+        <v>3/7/2026, 4:55:31 pm</v>
       </c>
       <c r="D109" t="str">
-        <v>7/5/2026, 12:06:36 am</v>
+        <v>3/7/2026, 4:55:36 pm</v>
       </c>
       <c r="E109" t="str">
         <v>Success</v>
@@ -2258,16 +2254,16 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>https://www.softwebsolutions.com/powerapps-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/power-bi-oee-dashboards/</v>
       </c>
       <c r="B110">
-        <v>5.18</v>
+        <v>6.16</v>
       </c>
       <c r="C110" t="str">
-        <v>7/5/2026, 12:06:41 am</v>
+        <v>3/7/2026, 4:55:41 pm</v>
       </c>
       <c r="D110" t="str">
-        <v>7/5/2026, 12:06:46 am</v>
+        <v>3/7/2026, 4:55:47 pm</v>
       </c>
       <c r="E110" t="str">
         <v>Success</v>
@@ -2275,16 +2271,16 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>https://www.softwebsolutions.com/predictive-analytics-services/</v>
+        <v>https://www.softwebsolutions.com/power-platform-consulting-services/</v>
       </c>
       <c r="B111">
-        <v>7.34</v>
+        <v>2.27</v>
       </c>
       <c r="C111" t="str">
-        <v>7/5/2026, 12:06:54 am</v>
+        <v>3/7/2026, 4:55:52 pm</v>
       </c>
       <c r="D111" t="str">
-        <v>7/5/2026, 12:07:02 am</v>
+        <v>3/7/2026, 4:55:54 pm</v>
       </c>
       <c r="E111" t="str">
         <v>Success</v>
@@ -2292,16 +2288,16 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>https://www.softwebsolutions.com/product-engineering-service/</v>
+        <v>https://www.softwebsolutions.com/powerapps-consulting-services/</v>
       </c>
       <c r="B112">
-        <v>5.47</v>
+        <v>2.86</v>
       </c>
       <c r="C112" t="str">
-        <v>7/5/2026, 12:07:08 am</v>
+        <v>3/7/2026, 4:55:58 pm</v>
       </c>
       <c r="D112" t="str">
-        <v>7/5/2026, 12:07:13 am</v>
+        <v>3/7/2026, 4:56:01 pm</v>
       </c>
       <c r="E112" t="str">
         <v>Success</v>
@@ -2309,16 +2305,16 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>https://www.softwebsolutions.com/product-information-management-system/</v>
+        <v>https://www.softwebsolutions.com/predictive-analytics-services/</v>
       </c>
       <c r="B113">
-        <v>1.43</v>
+        <v>5.16</v>
       </c>
       <c r="C113" t="str">
-        <v>7/5/2026, 12:07:19 am</v>
+        <v>3/7/2026, 4:56:05 pm</v>
       </c>
       <c r="D113" t="str">
-        <v>7/5/2026, 12:07:20 am</v>
+        <v>3/7/2026, 4:56:10 pm</v>
       </c>
       <c r="E113" t="str">
         <v>Success</v>
@@ -2326,16 +2322,16 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>https://www.softwebsolutions.com/</v>
+        <v>https://www.softwebsolutions.com/product-engineering-service/</v>
       </c>
       <c r="B114">
-        <v>7.21</v>
+        <v>4.93</v>
       </c>
       <c r="C114" t="str">
-        <v>7/5/2026, 12:00:42 am</v>
+        <v>3/7/2026, 4:56:14 pm</v>
       </c>
       <c r="D114" t="str">
-        <v>7/5/2026, 12:00:49 am</v>
+        <v>3/7/2026, 4:56:19 pm</v>
       </c>
       <c r="E114" t="str">
         <v>Success</v>
@@ -2343,16 +2339,16 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>https://www.softwebsolutions.com/about-softweb-solutions/</v>
+        <v>https://www.softwebsolutions.com/product-information-management-system/</v>
       </c>
       <c r="B115">
-        <v>6.49</v>
+        <v>5.16</v>
       </c>
       <c r="C115" t="str">
-        <v>7/5/2026, 12:00:57 am</v>
+        <v>3/7/2026, 4:56:23 pm</v>
       </c>
       <c r="D115" t="str">
-        <v>7/5/2026, 12:01:03 am</v>
+        <v>3/7/2026, 4:56:28 pm</v>
       </c>
       <c r="E115" t="str">
         <v>Success</v>
@@ -2360,16 +2356,16 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>https://www.softwebsolutions.com/adaptive-ai-development-company/</v>
+        <v>https://www.softwebsolutions.com/production-line-monitoring-solution/</v>
       </c>
       <c r="B116">
-        <v>5.03</v>
+        <v>0.86</v>
       </c>
       <c r="C116" t="str">
-        <v>7/5/2026, 12:01:10 am</v>
+        <v>3/7/2026, 4:48:28 pm</v>
       </c>
       <c r="D116" t="str">
-        <v>7/5/2026, 12:01:15 am</v>
+        <v>3/7/2026, 4:48:29 pm</v>
       </c>
       <c r="E116" t="str">
         <v>Success</v>
@@ -2377,16 +2373,16 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>https://www.softwebsolutions.com/agentforce-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/python-development-services/</v>
       </c>
       <c r="B117">
-        <v>1.82</v>
+        <v>1</v>
       </c>
       <c r="C117" t="str">
-        <v>7/5/2026, 12:01:22 am</v>
+        <v>3/7/2026, 4:48:34 pm</v>
       </c>
       <c r="D117" t="str">
-        <v>7/5/2026, 12:01:24 am</v>
+        <v>3/7/2026, 4:48:35 pm</v>
       </c>
       <c r="E117" t="str">
         <v>Success</v>
@@ -2394,16 +2390,16 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>https://www.softwebsolutions.com/agentic-ai-services/</v>
+        <v>https://www.softwebsolutions.com/quality-inspection-in-manufacturing/</v>
       </c>
       <c r="B118">
-        <v>5.78</v>
+        <v>4.98</v>
       </c>
       <c r="C118" t="str">
-        <v>7/5/2026, 12:01:31 am</v>
+        <v>3/7/2026, 4:48:42 pm</v>
       </c>
       <c r="D118" t="str">
-        <v>7/5/2026, 12:01:37 am</v>
+        <v>3/7/2026, 4:48:47 pm</v>
       </c>
       <c r="E118" t="str">
         <v>Success</v>
@@ -2411,16 +2407,16 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>https://www.softwebsolutions.com/ai-agent-development-company/</v>
+        <v>https://www.softwebsolutions.com/rag-as-a-service/</v>
       </c>
       <c r="B119">
-        <v>1.84</v>
+        <v>4.13</v>
       </c>
       <c r="C119" t="str">
-        <v>7/5/2026, 12:01:43 am</v>
+        <v>3/7/2026, 4:48:53 pm</v>
       </c>
       <c r="D119" t="str">
-        <v>7/5/2026, 12:01:45 am</v>
+        <v>3/7/2026, 4:48:57 pm</v>
       </c>
       <c r="E119" t="str">
         <v>Success</v>
@@ -2428,16 +2424,16 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>https://www.softwebsolutions.com/ai-anomaly-detection/</v>
+        <v>https://www.softwebsolutions.com/react-native-app-development-services/</v>
       </c>
       <c r="B120">
-        <v>0.96</v>
+        <v>5.89</v>
       </c>
       <c r="C120" t="str">
-        <v>7/5/2026, 12:01:52 am</v>
+        <v>3/7/2026, 4:49:02 pm</v>
       </c>
       <c r="D120" t="str">
-        <v>7/5/2026, 12:01:53 am</v>
+        <v>3/7/2026, 4:49:08 pm</v>
       </c>
       <c r="E120" t="str">
         <v>Success</v>
@@ -2445,16 +2441,16 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>https://www.softwebsolutions.com/ai-automation-testing-services/</v>
+        <v>https://www.softwebsolutions.com/reactjs-development-services/</v>
       </c>
       <c r="B121">
-        <v>0.84</v>
+        <v>6.01</v>
       </c>
       <c r="C121" t="str">
-        <v>7/5/2026, 12:01:59 am</v>
+        <v>3/7/2026, 4:49:13 pm</v>
       </c>
       <c r="D121" t="str">
-        <v>7/5/2026, 12:02:00 am</v>
+        <v>3/7/2026, 4:49:19 pm</v>
       </c>
       <c r="E121" t="str">
         <v>Success</v>
@@ -2462,16 +2458,16 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>https://www.softwebsolutions.com/ai-chatbot-development-company/</v>
+        <v>https://www.softwebsolutions.com/recommendation-system-development-services/</v>
       </c>
       <c r="B122">
-        <v>5.02</v>
+        <v>5.53</v>
       </c>
       <c r="C122" t="str">
-        <v>7/5/2026, 12:02:07 am</v>
+        <v>3/7/2026, 4:49:24 pm</v>
       </c>
       <c r="D122" t="str">
-        <v>7/5/2026, 12:02:12 am</v>
+        <v>3/7/2026, 4:49:30 pm</v>
       </c>
       <c r="E122" t="str">
         <v>Success</v>
@@ -2479,16 +2475,16 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>https://www.softwebsolutions.com/ai-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/salesforce-ai-consulting/</v>
       </c>
       <c r="B123">
-        <v>5.27</v>
+        <v>2.96</v>
       </c>
       <c r="C123" t="str">
-        <v>7/5/2026, 12:02:20 am</v>
+        <v>3/7/2026, 4:49:36 pm</v>
       </c>
       <c r="D123" t="str">
-        <v>7/5/2026, 12:02:25 am</v>
+        <v>3/7/2026, 4:49:39 pm</v>
       </c>
       <c r="E123" t="str">
         <v>Success</v>
@@ -2496,16 +2492,16 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>https://www.softwebsolutions.com/ai-defect-detection-visual-inspection/</v>
+        <v>https://www.softwebsolutions.com/salesforce-cloud-services/</v>
       </c>
       <c r="B124">
-        <v>4.92</v>
+        <v>5.81</v>
       </c>
       <c r="C124" t="str">
-        <v>7/5/2026, 12:02:31 am</v>
+        <v>3/7/2026, 4:49:45 pm</v>
       </c>
       <c r="D124" t="str">
-        <v>7/5/2026, 12:02:36 am</v>
+        <v>3/7/2026, 4:49:51 pm</v>
       </c>
       <c r="E124" t="str">
         <v>Success</v>
@@ -2513,16 +2509,16 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>https://www.softwebsolutions.com/ai-development-services/</v>
+        <v>https://www.softwebsolutions.com/salesforce-commerce-cloud-services/</v>
       </c>
       <c r="B125">
-        <v>5.05</v>
+        <v>6.3</v>
       </c>
       <c r="C125" t="str">
-        <v>7/5/2026, 12:02:44 am</v>
+        <v>3/7/2026, 4:49:58 pm</v>
       </c>
       <c r="D125" t="str">
-        <v>7/5/2026, 12:02:49 am</v>
+        <v>3/7/2026, 4:50:05 pm</v>
       </c>
       <c r="E125" t="str">
         <v>Success</v>
@@ -2530,16 +2526,16 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>https://www.softwebsolutions.com/ai-powered-inventory-management/</v>
+        <v>https://www.softwebsolutions.com/salesforce-consulting-services/</v>
       </c>
       <c r="B126">
-        <v>1.72</v>
+        <v>6.92</v>
       </c>
       <c r="C126" t="str">
-        <v>7/5/2026, 12:02:57 am</v>
+        <v>3/7/2026, 4:50:12 pm</v>
       </c>
       <c r="D126" t="str">
-        <v>7/5/2026, 12:02:58 am</v>
+        <v>3/7/2026, 4:50:18 pm</v>
       </c>
       <c r="E126" t="str">
         <v>Success</v>
@@ -2547,16 +2543,16 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>https://www.softwebsolutions.com/ai-prompt-engineering-services/</v>
+        <v>https://www.softwebsolutions.com/salesforce-data-cloud-services/</v>
       </c>
       <c r="B127">
-        <v>7.46</v>
+        <v>6.82</v>
       </c>
       <c r="C127" t="str">
-        <v>7/5/2026, 12:03:05 am</v>
+        <v>3/7/2026, 4:50:26 pm</v>
       </c>
       <c r="D127" t="str">
-        <v>7/5/2026, 12:03:13 am</v>
+        <v>3/7/2026, 4:50:33 pm</v>
       </c>
       <c r="E127" t="str">
         <v>Success</v>
@@ -2564,16 +2560,16 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>https://www.softwebsolutions.com/aiops-solutions/</v>
+        <v>https://www.softwebsolutions.com/salesforce-development-services/</v>
       </c>
       <c r="B128">
-        <v>1.47</v>
+        <v>10.55</v>
       </c>
       <c r="C128" t="str">
-        <v>7/5/2026, 12:03:18 am</v>
+        <v>3/7/2026, 4:50:45 pm</v>
       </c>
       <c r="D128" t="str">
-        <v>7/5/2026, 12:03:19 am</v>
+        <v>3/7/2026, 4:50:55 pm</v>
       </c>
       <c r="E128" t="str">
         <v>Success</v>
@@ -2581,16 +2577,16 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>https://www.softwebsolutions.com/application-managed-services/</v>
+        <v>https://www.softwebsolutions.com/salesforce-experience-cloud-services/</v>
       </c>
       <c r="B129">
-        <v>9.18</v>
+        <v>2.93</v>
       </c>
       <c r="C129" t="str">
-        <v>7/5/2026, 12:03:25 am</v>
+        <v>3/7/2026, 4:51:14 pm</v>
       </c>
       <c r="D129" t="str">
-        <v>7/5/2026, 12:03:35 am</v>
+        <v>3/7/2026, 4:51:17 pm</v>
       </c>
       <c r="E129" t="str">
         <v>Success</v>
@@ -2598,16 +2594,16 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>https://www.softwebsolutions.com/automated-data-capture-solutions/</v>
+        <v>https://www.softwebsolutions.com/salesforce-implementation-services/</v>
       </c>
       <c r="B130">
-        <v>4.82</v>
+        <v>5.73</v>
       </c>
       <c r="C130" t="str">
-        <v>7/5/2026, 12:03:41 am</v>
+        <v>3/7/2026, 4:51:25 pm</v>
       </c>
       <c r="D130" t="str">
-        <v>7/5/2026, 12:03:46 am</v>
+        <v>3/7/2026, 4:51:30 pm</v>
       </c>
       <c r="E130" t="str">
         <v>Success</v>
@@ -2615,16 +2611,16 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>https://www.softwebsolutions.com/automated-quality-control-inspection-with-ai/</v>
+        <v>https://www.softwebsolutions.com/salesforce-integration-services/</v>
       </c>
       <c r="B131">
-        <v>5.64</v>
+        <v>2.87</v>
       </c>
       <c r="C131" t="str">
-        <v>7/5/2026, 12:03:51 am</v>
+        <v>3/7/2026, 4:51:39 pm</v>
       </c>
       <c r="D131" t="str">
-        <v>7/5/2026, 12:03:57 am</v>
+        <v>3/7/2026, 4:51:42 pm</v>
       </c>
       <c r="E131" t="str">
         <v>Success</v>
@@ -2632,16 +2628,16 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>https://www.softwebsolutions.com/autonomous-ai-agents-development/</v>
+        <v>https://www.softwebsolutions.com/salesforce-migration-services/</v>
       </c>
       <c r="B132">
-        <v>5.93</v>
+        <v>5.89</v>
       </c>
       <c r="C132" t="str">
-        <v>7/5/2026, 12:04:04 am</v>
+        <v>3/7/2026, 4:51:48 pm</v>
       </c>
       <c r="D132" t="str">
-        <v>7/5/2026, 12:04:10 am</v>
+        <v>3/7/2026, 4:51:54 pm</v>
       </c>
       <c r="E132" t="str">
         <v>Success</v>
@@ -2649,16 +2645,16 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>https://www.softwebsolutions.com/aws-cloud-migration-services/</v>
+        <v>https://www.softwebsolutions.com/salesforce-revenue-cloud-advanced/</v>
       </c>
       <c r="B133">
-        <v>1.23</v>
+        <v>5.67</v>
       </c>
       <c r="C133" t="str">
-        <v>7/5/2026, 12:04:16 am</v>
+        <v>3/7/2026, 4:52:00 pm</v>
       </c>
       <c r="D133" t="str">
-        <v>7/5/2026, 12:04:18 am</v>
+        <v>3/7/2026, 4:52:06 pm</v>
       </c>
       <c r="E133" t="str">
         <v>Success</v>
@@ -2666,16 +2662,16 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>https://www.softwebsolutions.com/aws-data-analytics-consulting/</v>
+        <v>https://www.softwebsolutions.com/salesforce-revenue-cloud-services/</v>
       </c>
       <c r="B134">
-        <v>1.18</v>
+        <v>7.36</v>
       </c>
       <c r="C134" t="str">
-        <v>7/5/2026, 12:04:24 am</v>
+        <v>3/7/2026, 4:52:11 pm</v>
       </c>
       <c r="D134" t="str">
-        <v>7/5/2026, 12:04:25 am</v>
+        <v>3/7/2026, 4:52:18 pm</v>
       </c>
       <c r="E134" t="str">
         <v>Success</v>
@@ -2683,16 +2679,16 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>https://www.softwebsolutions.com/aws-sagemaker-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/salesforce-sales-cloud-services/</v>
       </c>
       <c r="B135">
-        <v>1.16</v>
+        <v>5.99</v>
       </c>
       <c r="C135" t="str">
-        <v>7/5/2026, 12:04:32 am</v>
+        <v>3/7/2026, 4:52:24 pm</v>
       </c>
       <c r="D135" t="str">
-        <v>7/5/2026, 12:04:33 am</v>
+        <v>3/7/2026, 4:52:29 pm</v>
       </c>
       <c r="E135" t="str">
         <v>Success</v>
@@ -2700,16 +2696,16 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>https://www.softwebsolutions.com/aws-services/</v>
+        <v>https://www.softwebsolutions.com/semiconductor/</v>
       </c>
       <c r="B136">
-        <v>1.62</v>
+        <v>1.15</v>
       </c>
       <c r="C136" t="str">
-        <v>7/5/2026, 12:04:41 am</v>
+        <v>3/7/2026, 4:52:35 pm</v>
       </c>
       <c r="D136" t="str">
-        <v>7/5/2026, 12:04:42 am</v>
+        <v>3/7/2026, 4:52:37 pm</v>
       </c>
       <c r="E136" t="str">
         <v>Success</v>
@@ -2717,16 +2713,16 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>https://www.softwebsolutions.com/azure-ai-services/</v>
+        <v>https://www.softwebsolutions.com/sharepoint-consulting-services/</v>
       </c>
       <c r="B137">
-        <v>1.22</v>
+        <v>6.2</v>
       </c>
       <c r="C137" t="str">
-        <v>7/5/2026, 12:04:49 am</v>
+        <v>3/7/2026, 4:52:44 pm</v>
       </c>
       <c r="D137" t="str">
-        <v>7/5/2026, 12:04:50 am</v>
+        <v>3/7/2026, 4:52:50 pm</v>
       </c>
       <c r="E137" t="str">
         <v>Success</v>
@@ -2734,16 +2730,16 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>https://www.softwebsolutions.com/azure-cloud-service/</v>
+        <v>https://www.softwebsolutions.com/simple-reflex-ai-agents/</v>
       </c>
       <c r="B138">
-        <v>5.57</v>
+        <v>5.82</v>
       </c>
       <c r="C138" t="str">
-        <v>7/5/2026, 12:04:57 am</v>
+        <v>3/7/2026, 4:52:56 pm</v>
       </c>
       <c r="D138" t="str">
-        <v>7/5/2026, 12:05:03 am</v>
+        <v>3/7/2026, 4:53:02 pm</v>
       </c>
       <c r="E138" t="str">
         <v>Success</v>
@@ -2751,16 +2747,16 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>https://www.softwebsolutions.com/azure-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/sitecore-implementation/</v>
       </c>
       <c r="B139">
-        <v>1.81</v>
+        <v>7.08</v>
       </c>
       <c r="C139" t="str">
-        <v>7/5/2026, 12:05:10 am</v>
+        <v>3/7/2026, 4:53:09 pm</v>
       </c>
       <c r="D139" t="str">
-        <v>7/5/2026, 12:05:12 am</v>
+        <v>3/7/2026, 4:53:16 pm</v>
       </c>
       <c r="E139" t="str">
         <v>Success</v>
@@ -2768,16 +2764,16 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>https://www.softwebsolutions.com/azure-data-services/</v>
+        <v>https://www.softwebsolutions.com/sitecore-managed-services/</v>
       </c>
       <c r="B140">
-        <v>1.08</v>
+        <v>7.78</v>
       </c>
       <c r="C140" t="str">
-        <v>7/5/2026, 12:05:18 am</v>
+        <v>3/7/2026, 4:53:25 pm</v>
       </c>
       <c r="D140" t="str">
-        <v>7/5/2026, 12:05:19 am</v>
+        <v>3/7/2026, 4:53:33 pm</v>
       </c>
       <c r="E140" t="str">
         <v>Success</v>
@@ -2785,16 +2781,16 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>https://www.softwebsolutions.com/azure-devops-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/snowflake-consulting-services/</v>
       </c>
       <c r="B141">
-        <v>5.29</v>
+        <v>3.35</v>
       </c>
       <c r="C141" t="str">
-        <v>7/5/2026, 12:05:27 am</v>
+        <v>3/7/2026, 4:53:39 pm</v>
       </c>
       <c r="D141" t="str">
-        <v>7/5/2026, 12:05:33 am</v>
+        <v>3/7/2026, 4:53:42 pm</v>
       </c>
       <c r="E141" t="str">
         <v>Success</v>
@@ -2802,16 +2798,16 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>https://www.softwebsolutions.com/big-data-services/</v>
+        <v>https://www.softwebsolutions.com/solutions/</v>
       </c>
       <c r="B142">
-        <v>6.13</v>
+        <v>5.86</v>
       </c>
       <c r="C142" t="str">
-        <v>7/5/2026, 12:05:39 am</v>
+        <v>3/7/2026, 4:53:49 pm</v>
       </c>
       <c r="D142" t="str">
-        <v>7/5/2026, 12:05:45 am</v>
+        <v>3/7/2026, 4:53:54 pm</v>
       </c>
       <c r="E142" t="str">
         <v>Success</v>
@@ -2819,16 +2815,16 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>https://www.softwebsolutions.com/business-intelligence-consulting/</v>
+        <v>https://www.softwebsolutions.com/supply-chain-automation-solution/</v>
       </c>
       <c r="B143">
-        <v>6.96</v>
+        <v>5.82</v>
       </c>
       <c r="C143" t="str">
-        <v>7/5/2026, 12:05:50 am</v>
+        <v>3/7/2026, 4:54:01 pm</v>
       </c>
       <c r="D143" t="str">
-        <v>7/5/2026, 12:05:57 am</v>
+        <v>3/7/2026, 4:54:07 pm</v>
       </c>
       <c r="E143" t="str">
         <v>Success</v>
@@ -2836,16 +2832,16 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>https://www.softwebsolutions.com/business-process-automation-services/</v>
+        <v>https://www.softwebsolutions.com/supply-chain-bot-development/</v>
       </c>
       <c r="B144">
-        <v>7.59</v>
+        <v>5.83</v>
       </c>
       <c r="C144" t="str">
-        <v>7/5/2026, 12:06:02 am</v>
+        <v>3/7/2026, 4:54:14 pm</v>
       </c>
       <c r="D144" t="str">
-        <v>7/5/2026, 12:06:09 am</v>
+        <v>3/7/2026, 4:54:20 pm</v>
       </c>
       <c r="E144" t="str">
         <v>Success</v>
@@ -2853,16 +2849,16 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>https://www.softwebsolutions.com/client-testimonial/</v>
+        <v>https://www.softwebsolutions.com/supply-chain/</v>
       </c>
       <c r="B145">
-        <v>4.91</v>
+        <v>4.5</v>
       </c>
       <c r="C145" t="str">
-        <v>7/5/2026, 12:06:15 am</v>
+        <v>3/7/2026, 4:54:27 pm</v>
       </c>
       <c r="D145" t="str">
-        <v>7/5/2026, 12:06:20 am</v>
+        <v>3/7/2026, 4:54:31 pm</v>
       </c>
       <c r="E145" t="str">
         <v>Success</v>
@@ -2870,16 +2866,16 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>https://www.softwebsolutions.com/cloud-application-development-services/</v>
+        <v>https://www.softwebsolutions.com/surface-defect-detection/</v>
       </c>
       <c r="B146">
-        <v>13.24</v>
+        <v>6.92</v>
       </c>
       <c r="C146" t="str">
-        <v>7/5/2026, 12:06:26 am</v>
+        <v>3/7/2026, 4:54:40 pm</v>
       </c>
       <c r="D146" t="str">
-        <v>7/5/2026, 12:06:39 am</v>
+        <v>3/7/2026, 4:54:47 pm</v>
       </c>
       <c r="E146" t="str">
         <v>Success</v>
@@ -2887,16 +2883,16 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>https://www.softwebsolutions.com/cloud-consulting-services/</v>
+        <v>https://www.softwebsolutions.com/tableau-consulting-services/</v>
       </c>
       <c r="B147">
-        <v>5.37</v>
+        <v>5.84</v>
       </c>
       <c r="C147" t="str">
-        <v>7/5/2026, 12:06:44 am</v>
+        <v>3/7/2026, 4:54:58 pm</v>
       </c>
       <c r="D147" t="str">
-        <v>7/5/2026, 12:06:49 am</v>
+        <v>3/7/2026, 4:55:04 pm</v>
       </c>
       <c r="E147" t="str">
         <v>Success</v>
@@ -2904,16 +2900,16 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>https://www.softwebsolutions.com/cloud-managed-services/</v>
+        <v>https://www.softwebsolutions.com/vision-based-eol-detection/</v>
       </c>
       <c r="B148">
-        <v>6.05</v>
+        <v>6.41</v>
       </c>
       <c r="C148" t="str">
-        <v>7/5/2026, 12:06:55 am</v>
+        <v>3/7/2026, 4:55:11 pm</v>
       </c>
       <c r="D148" t="str">
-        <v>7/5/2026, 12:07:01 am</v>
+        <v>3/7/2026, 4:55:18 pm</v>
       </c>
       <c r="E148" t="str">
         <v>Success</v>
@@ -2921,16 +2917,16 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>https://www.softwebsolutions.com/cloud-migration-services/</v>
+        <v>https://www.softwebsolutions.com/wafer-defect-detection/</v>
       </c>
       <c r="B149">
-        <v>2.01</v>
+        <v>5.14</v>
       </c>
       <c r="C149" t="str">
-        <v>7/5/2026, 12:07:08 am</v>
+        <v>3/7/2026, 4:55:23 pm</v>
       </c>
       <c r="D149" t="str">
-        <v>7/5/2026, 12:07:10 am</v>
+        <v>3/7/2026, 4:55:28 pm</v>
       </c>
       <c r="E149" t="str">
         <v>Success</v>
@@ -2938,16 +2934,16 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>https://www.softwebsolutions.com/cloud-transformation-services/</v>
+        <v>https://www.softwebsolutions.com/web-application-development/</v>
       </c>
       <c r="B150">
-        <v>2</v>
+        <v>6.13</v>
       </c>
       <c r="C150" t="str">
-        <v>7/5/2026, 12:07:17 am</v>
+        <v>3/7/2026, 4:55:32 pm</v>
       </c>
       <c r="D150" t="str">
-        <v>7/5/2026, 12:07:19 am</v>
+        <v>3/7/2026, 4:55:39 pm</v>
       </c>
       <c r="E150" t="str">
         <v>Success</v>
@@ -2955,16 +2951,16 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>https://www.softwebsolutions.com/computer-vision/</v>
+        <v>https://www.softwebsolutions.com/wordpress-development-services/</v>
       </c>
       <c r="B151">
-        <v>1.89</v>
+        <v>1.76</v>
       </c>
       <c r="C151" t="str">
-        <v>7/5/2026, 12:07:24 am</v>
+        <v>3/7/2026, 4:55:44 pm</v>
       </c>
       <c r="D151" t="str">
-        <v>7/5/2026, 12:07:26 am</v>
+        <v>3/7/2026, 4:55:46 pm</v>
       </c>
       <c r="E151" t="str">
         <v>Success</v>

</xml_diff>